<commit_message>
data: update 2026-04-27 10:46
</commit_message>
<xml_diff>
--- a/output/oem_master.xlsx
+++ b/output/oem_master.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="manual_data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="manual_data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,82 +459,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Maker</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Model / Type</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Part to be lubricated</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Lubricant</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>source_file</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>source_sheet</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I356"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -14438,6 +14365,123 @@
       <c r="H356" s="2" t="inlineStr"/>
       <c r="I356" s="2" t="inlineStr"/>
     </row>
+    <row r="357">
+      <c r="A357" s="4" t="inlineStr">
+        <is>
+          <t>DIESEL GENERATOR ENGINE</t>
+        </is>
+      </c>
+      <c r="B357" s="4" t="inlineStr">
+        <is>
+          <t>HIMSEN</t>
+        </is>
+      </c>
+      <c r="C357" s="4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D357" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; CRANKCASE (LNG)</t>
+        </is>
+      </c>
+      <c r="E357" s="4" t="inlineStr">
+        <is>
+          <t>AURELIA NGX 40</t>
+        </is>
+      </c>
+      <c r="F357" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G357" s="5" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="H357" s="4" t="inlineStr"/>
+      <c r="I357" s="4" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>DIESEL GENERATOR ENGINE</t>
+        </is>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>WARTSILA</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; CRANKCASE (LNG)</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>AURELIA NGX 40</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="H358" s="2" t="inlineStr"/>
+      <c r="I358" s="2" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="inlineStr">
+        <is>
+          <t>DIESEL GENERATOR ENGINE</t>
+        </is>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>EVERLLENCE</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; CRANKCASE (LNG)</t>
+        </is>
+      </c>
+      <c r="E359" s="4" t="inlineStr">
+        <is>
+          <t>AURELIA NGX 40</t>
+        </is>
+      </c>
+      <c r="F359" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G359" s="5" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="H359" s="4" t="inlineStr"/>
+      <c r="I359" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update 2026-04-30 11:51
</commit_message>
<xml_diff>
--- a/output/oem_master.xlsx
+++ b/output/oem_master.xlsx
@@ -22700,7 +22700,7 @@
       </c>
       <c r="D581" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature         -20°C…+5°C</t>
+          <t>Ambient Temperature -20°C…+5°C</t>
         </is>
       </c>
       <c r="E581" s="4" t="inlineStr">
@@ -22739,7 +22739,7 @@
       </c>
       <c r="D582" s="2" t="inlineStr">
         <is>
-          <t>Ambient Temperature         5°C…40°C</t>
+          <t>Ambient Temperature 5°C…40°C</t>
         </is>
       </c>
       <c r="E582" s="2" t="inlineStr">
@@ -22778,7 +22778,7 @@
       </c>
       <c r="D583" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature         30°C…65°C</t>
+          <t>Ambient Temperature 30°C…65°C</t>
         </is>
       </c>
       <c r="E583" s="4" t="inlineStr">
@@ -23517,8 +23517,7 @@
       </c>
       <c r="D604" s="2" t="inlineStr">
         <is>
-          <t>Ambient Temperature
- -20°C…10°C</t>
+          <t>Ambient Temperature -20°C…10°C</t>
         </is>
       </c>
       <c r="E604" s="2" t="inlineStr">
@@ -23557,8 +23556,7 @@
       </c>
       <c r="D605" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature
- 10°C…50°C</t>
+          <t>Ambient Temperature 10°C…50°C</t>
         </is>
       </c>
       <c r="E605" s="4" t="inlineStr">
@@ -23597,8 +23595,7 @@
       </c>
       <c r="D606" s="2" t="inlineStr">
         <is>
-          <t>Ambient Temperature
- -20°C…10°C</t>
+          <t>Ambient Temperature -20°C…10°C</t>
         </is>
       </c>
       <c r="E606" s="2" t="inlineStr">
@@ -23637,8 +23634,7 @@
       </c>
       <c r="D607" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature
- 10°C…50°C</t>
+          <t>Ambient Temperature 10°C…50°C</t>
         </is>
       </c>
       <c r="E607" s="4" t="inlineStr">
@@ -28701,7 +28697,7 @@
       <c r="C748" s="2" t="inlineStr"/>
       <c r="D748" s="2" t="inlineStr">
         <is>
-          <t>Initial Fill  - Viscosity 50/55cSt at 40°C</t>
+          <t>Initial Fill - Viscosity 50/55cSt at 40°C</t>
         </is>
       </c>
       <c r="E748" s="2" t="inlineStr">
@@ -28802,8 +28798,7 @@
       </c>
       <c r="D751" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature
-0…15°C</t>
+          <t>Ambient Temperature 0…15°C</t>
         </is>
       </c>
       <c r="E751" s="4" t="inlineStr">
@@ -28842,8 +28837,7 @@
       </c>
       <c r="D752" s="2" t="inlineStr">
         <is>
-          <t>Ambient Temperature
-15…25°C</t>
+          <t>Ambient Temperature 15…25°C</t>
         </is>
       </c>
       <c r="E752" s="2" t="inlineStr">
@@ -28882,8 +28876,7 @@
       </c>
       <c r="D753" s="4" t="inlineStr">
         <is>
-          <t>Ambient Temperature
-25…35°C</t>
+          <t>Ambient Temperature 25…35°C</t>
         </is>
       </c>
       <c r="E753" s="4" t="inlineStr">
@@ -28922,8 +28915,7 @@
       </c>
       <c r="D754" s="2" t="inlineStr">
         <is>
-          <t>Ambient Temperature
-35…45°C</t>
+          <t>Ambient Temperature 35…45°C</t>
         </is>
       </c>
       <c r="E754" s="2" t="inlineStr">
@@ -32032,7 +32024,7 @@
       <c r="C841" s="4" t="inlineStr"/>
       <c r="D841" s="4" t="inlineStr">
         <is>
-          <t>Initial Fill  - Viscosity 50/55cSt at 40°C</t>
+          <t>Initial Fill - Viscosity 50/55cSt at 40°C</t>
         </is>
       </c>
       <c r="E841" s="4" t="inlineStr">
@@ -32451,7 +32443,7 @@
       </c>
       <c r="C853" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-CFC</t>
         </is>
       </c>
       <c r="D853" s="4" t="inlineStr">
@@ -32490,7 +32482,7 @@
       </c>
       <c r="C854" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HCFC</t>
         </is>
       </c>
       <c r="D854" s="2" t="inlineStr">
@@ -32529,7 +32521,7 @@
       </c>
       <c r="C855" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HCFC</t>
         </is>
       </c>
       <c r="D855" s="4" t="inlineStr">
@@ -32568,7 +32560,7 @@
       </c>
       <c r="C856" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HCFC</t>
         </is>
       </c>
       <c r="D856" s="2" t="inlineStr">
@@ -32607,7 +32599,7 @@
       </c>
       <c r="C857" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HFC</t>
         </is>
       </c>
       <c r="D857" s="4" t="inlineStr">
@@ -32646,7 +32638,7 @@
       </c>
       <c r="C858" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D858" s="2" t="inlineStr">
@@ -32685,7 +32677,7 @@
       </c>
       <c r="C859" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D859" s="4" t="inlineStr">
@@ -32724,7 +32716,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -32763,7 +32755,7 @@
       </c>
       <c r="C861" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A-HFC</t>
         </is>
       </c>
       <c r="D861" s="4" t="inlineStr"/>
@@ -32798,7 +32790,7 @@
       </c>
       <c r="C862" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B-HFC</t>
         </is>
       </c>
       <c r="D862" s="2" t="inlineStr"/>
@@ -32833,7 +32825,7 @@
       </c>
       <c r="C863" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C-HFC</t>
         </is>
       </c>
       <c r="D863" s="4" t="inlineStr"/>
@@ -32868,7 +32860,7 @@
       </c>
       <c r="C864" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>D-HFC</t>
         </is>
       </c>
       <c r="D864" s="2" t="inlineStr"/>
@@ -32903,7 +32895,7 @@
       </c>
       <c r="C865" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F-HFC</t>
         </is>
       </c>
       <c r="D865" s="4" t="inlineStr"/>
@@ -32938,7 +32930,7 @@
       </c>
       <c r="C866" s="2" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Q-HFC</t>
         </is>
       </c>
       <c r="D866" s="2" t="inlineStr"/>
@@ -32973,7 +32965,7 @@
       </c>
       <c r="C867" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-HFC</t>
         </is>
       </c>
       <c r="D867" s="4" t="inlineStr"/>
@@ -33008,7 +33000,7 @@
       </c>
       <c r="C868" s="2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>V-HFC</t>
         </is>
       </c>
       <c r="D868" s="2" t="inlineStr"/>
@@ -33043,7 +33035,7 @@
       </c>
       <c r="C869" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>Z-HFC</t>
         </is>
       </c>
       <c r="D869" s="4" t="inlineStr"/>
@@ -33078,7 +33070,7 @@
       </c>
       <c r="C870" s="2" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>W-HFC</t>
         </is>
       </c>
       <c r="D870" s="2" t="inlineStr"/>
@@ -33113,7 +33105,7 @@
       </c>
       <c r="C871" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HFC</t>
         </is>
       </c>
       <c r="D871" s="4" t="inlineStr"/>
@@ -33148,7 +33140,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HFC</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr"/>
@@ -33183,7 +33175,7 @@
       </c>
       <c r="C873" s="4" t="inlineStr">
         <is>
-          <t>Serie 6</t>
+          <t>Serie 6-R717 (NH3)</t>
         </is>
       </c>
       <c r="D873" s="4" t="inlineStr">
@@ -33222,7 +33214,7 @@
       </c>
       <c r="C874" s="2" t="inlineStr">
         <is>
-          <t>Serie 6</t>
+          <t>Serie 6-HCFC</t>
         </is>
       </c>
       <c r="D874" s="2" t="inlineStr">
@@ -33261,7 +33253,7 @@
       </c>
       <c r="C875" s="4" t="inlineStr">
         <is>
-          <t>Serie 6</t>
+          <t>Serie 6-HFC</t>
         </is>
       </c>
       <c r="D875" s="4" t="inlineStr">
@@ -33300,7 +33292,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>Serie 10</t>
+          <t>Serie 10-R717 (NH3)</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -33339,7 +33331,7 @@
       </c>
       <c r="C877" s="4" t="inlineStr">
         <is>
-          <t>Serie 10</t>
+          <t>Serie 10-HCFC</t>
         </is>
       </c>
       <c r="D877" s="4" t="inlineStr">
@@ -33378,7 +33370,7 @@
       </c>
       <c r="C878" s="2" t="inlineStr">
         <is>
-          <t>Serie 10</t>
+          <t>Serie 10-HFC</t>
         </is>
       </c>
       <c r="D878" s="2" t="inlineStr">
@@ -33417,7 +33409,7 @@
       </c>
       <c r="C879" s="4" t="inlineStr">
         <is>
-          <t>Serie 12/12E</t>
+          <t>Serie 12/12E-R717 (NH3)</t>
         </is>
       </c>
       <c r="D879" s="4" t="inlineStr">
@@ -33456,7 +33448,7 @@
       </c>
       <c r="C880" s="2" t="inlineStr">
         <is>
-          <t>Serie 12/12E</t>
+          <t>Serie 12/12E-HCFC</t>
         </is>
       </c>
       <c r="D880" s="2" t="inlineStr">
@@ -33495,7 +33487,7 @@
       </c>
       <c r="C881" s="4" t="inlineStr">
         <is>
-          <t>Serie 12/12E</t>
+          <t>Serie 12/12E-HFC</t>
         </is>
       </c>
       <c r="D881" s="4" t="inlineStr">
@@ -33534,7 +33526,7 @@
       </c>
       <c r="C882" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D882" s="2" t="inlineStr">
@@ -33573,7 +33565,7 @@
       </c>
       <c r="C883" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D883" s="4" t="inlineStr">
@@ -33612,7 +33604,7 @@
       </c>
       <c r="C884" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R717 (NH3)</t>
         </is>
       </c>
       <c r="D884" s="2" t="inlineStr">
@@ -33651,7 +33643,7 @@
       </c>
       <c r="C885" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-R22 (HCFC)</t>
         </is>
       </c>
       <c r="D885" s="4" t="inlineStr"/>
@@ -33686,7 +33678,7 @@
       </c>
       <c r="C886" s="2" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-HFC</t>
         </is>
       </c>
       <c r="D886" s="2" t="inlineStr">
@@ -33725,7 +33717,7 @@
       </c>
       <c r="C887" s="4" t="inlineStr">
         <is>
-          <t>all types</t>
+          <t>all types-Natural Gas</t>
         </is>
       </c>
       <c r="D887" s="4" t="inlineStr"/>
@@ -33760,7 +33752,7 @@
       </c>
       <c r="C888" s="2" t="inlineStr">
         <is>
-          <t>XRV</t>
+          <t>XRV-HFC</t>
         </is>
       </c>
       <c r="D888" s="2" t="inlineStr">
@@ -33799,7 +33791,7 @@
       </c>
       <c r="C889" s="4" t="inlineStr">
         <is>
-          <t>XRV</t>
+          <t>XRV-R717 (NH3)</t>
         </is>
       </c>
       <c r="D889" s="4" t="inlineStr"/>
@@ -33834,7 +33826,7 @@
       </c>
       <c r="C890" s="2" t="inlineStr">
         <is>
-          <t>WRV</t>
+          <t>WRV-HFC</t>
         </is>
       </c>
       <c r="D890" s="2" t="inlineStr">
@@ -33873,7 +33865,7 @@
       </c>
       <c r="C891" s="4" t="inlineStr">
         <is>
-          <t>WRV</t>
+          <t>WRV-R717 (NH3)</t>
         </is>
       </c>
       <c r="D891" s="4" t="inlineStr"/>
@@ -33906,7 +33898,11 @@
           <t>York (Johnson Controls)</t>
         </is>
       </c>
-      <c r="C892" s="2" t="inlineStr"/>
+      <c r="C892" s="2" t="inlineStr">
+        <is>
+          <t>HFC</t>
+        </is>
+      </c>
       <c r="D892" s="2" t="inlineStr">
         <is>
           <t>Type and Grade chosen according to operating conditions</t>
@@ -33941,7 +33937,11 @@
           <t>York (Johnson Controls)</t>
         </is>
       </c>
-      <c r="C893" s="4" t="inlineStr"/>
+      <c r="C893" s="4" t="inlineStr">
+        <is>
+          <t>HFC</t>
+        </is>
+      </c>
       <c r="D893" s="4" t="inlineStr">
         <is>
           <t>Type and Grade chosen according to operating conditions</t>
@@ -36086,7 +36086,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>BWPX</t>
+          <t>BWPX-307</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr"/>
@@ -36121,7 +36121,7 @@
       </c>
       <c r="C963" s="4" t="inlineStr">
         <is>
-          <t>BWPX</t>
+          <t>BWPX-307</t>
         </is>
       </c>
       <c r="D963" s="4" t="inlineStr"/>
@@ -36156,7 +36156,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>BWPX</t>
+          <t>BWPX-307</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr"/>
@@ -36191,7 +36191,7 @@
       </c>
       <c r="C965" s="4" t="inlineStr">
         <is>
-          <t>BWPX</t>
+          <t>BWPX-307</t>
         </is>
       </c>
       <c r="D965" s="4" t="inlineStr"/>
@@ -36226,7 +36226,7 @@
       </c>
       <c r="C966" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-605</t>
         </is>
       </c>
       <c r="D966" s="2" t="inlineStr"/>
@@ -36261,7 +36261,7 @@
       </c>
       <c r="C967" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-605</t>
         </is>
       </c>
       <c r="D967" s="4" t="inlineStr"/>
@@ -36296,7 +36296,7 @@
       </c>
       <c r="C968" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-605</t>
         </is>
       </c>
       <c r="D968" s="2" t="inlineStr"/>
@@ -36331,7 +36331,7 @@
       </c>
       <c r="C969" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-605</t>
         </is>
       </c>
       <c r="D969" s="4" t="inlineStr"/>
@@ -36366,7 +36366,7 @@
       </c>
       <c r="C970" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-605</t>
         </is>
       </c>
       <c r="D970" s="2" t="inlineStr"/>
@@ -36401,7 +36401,7 @@
       </c>
       <c r="C971" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-607</t>
         </is>
       </c>
       <c r="D971" s="4" t="inlineStr"/>
@@ -36436,7 +36436,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-607</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr"/>
@@ -36471,7 +36471,7 @@
       </c>
       <c r="C973" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-607</t>
         </is>
       </c>
       <c r="D973" s="4" t="inlineStr"/>
@@ -36506,7 +36506,7 @@
       </c>
       <c r="C974" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-607</t>
         </is>
       </c>
       <c r="D974" s="2" t="inlineStr"/>
@@ -36541,7 +36541,7 @@
       </c>
       <c r="C975" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-607</t>
         </is>
       </c>
       <c r="D975" s="4" t="inlineStr"/>
@@ -36576,7 +36576,7 @@
       </c>
       <c r="C976" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-609</t>
         </is>
       </c>
       <c r="D976" s="2" t="inlineStr"/>
@@ -36611,7 +36611,7 @@
       </c>
       <c r="C977" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-609</t>
         </is>
       </c>
       <c r="D977" s="4" t="inlineStr"/>
@@ -36646,7 +36646,7 @@
       </c>
       <c r="C978" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-609</t>
         </is>
       </c>
       <c r="D978" s="2" t="inlineStr"/>
@@ -36681,7 +36681,7 @@
       </c>
       <c r="C979" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-609</t>
         </is>
       </c>
       <c r="D979" s="4" t="inlineStr"/>
@@ -36716,7 +36716,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-609</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr"/>
@@ -36751,7 +36751,7 @@
       </c>
       <c r="C981" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-610</t>
         </is>
       </c>
       <c r="D981" s="4" t="inlineStr"/>
@@ -36786,7 +36786,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-610</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr"/>
@@ -36821,7 +36821,7 @@
       </c>
       <c r="C983" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-610</t>
         </is>
       </c>
       <c r="D983" s="4" t="inlineStr"/>
@@ -36856,7 +36856,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-610</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr"/>
@@ -36891,7 +36891,7 @@
       </c>
       <c r="C985" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-610</t>
         </is>
       </c>
       <c r="D985" s="4" t="inlineStr"/>
@@ -36926,7 +36926,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-611</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr"/>
@@ -36961,7 +36961,7 @@
       </c>
       <c r="C987" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-611</t>
         </is>
       </c>
       <c r="D987" s="4" t="inlineStr"/>
@@ -36996,7 +36996,7 @@
       </c>
       <c r="C988" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-611</t>
         </is>
       </c>
       <c r="D988" s="2" t="inlineStr"/>
@@ -37031,7 +37031,7 @@
       </c>
       <c r="C989" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-611</t>
         </is>
       </c>
       <c r="D989" s="4" t="inlineStr"/>
@@ -37066,7 +37066,7 @@
       </c>
       <c r="C990" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-611</t>
         </is>
       </c>
       <c r="D990" s="2" t="inlineStr"/>
@@ -37101,7 +37101,7 @@
       </c>
       <c r="C991" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-613</t>
         </is>
       </c>
       <c r="D991" s="4" t="inlineStr"/>
@@ -37136,7 +37136,7 @@
       </c>
       <c r="C992" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-613</t>
         </is>
       </c>
       <c r="D992" s="2" t="inlineStr"/>
@@ -37171,7 +37171,7 @@
       </c>
       <c r="C993" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-613</t>
         </is>
       </c>
       <c r="D993" s="4" t="inlineStr"/>
@@ -37206,7 +37206,7 @@
       </c>
       <c r="C994" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-613</t>
         </is>
       </c>
       <c r="D994" s="2" t="inlineStr"/>
@@ -37241,7 +37241,7 @@
       </c>
       <c r="C995" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-613</t>
         </is>
       </c>
       <c r="D995" s="4" t="inlineStr"/>
@@ -37276,7 +37276,7 @@
       </c>
       <c r="C996" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-614</t>
         </is>
       </c>
       <c r="D996" s="2" t="inlineStr"/>
@@ -37311,7 +37311,7 @@
       </c>
       <c r="C997" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-614</t>
         </is>
       </c>
       <c r="D997" s="4" t="inlineStr"/>
@@ -37346,7 +37346,7 @@
       </c>
       <c r="C998" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-614</t>
         </is>
       </c>
       <c r="D998" s="2" t="inlineStr"/>
@@ -37381,7 +37381,7 @@
       </c>
       <c r="C999" s="4" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-614</t>
         </is>
       </c>
       <c r="D999" s="4" t="inlineStr"/>
@@ -37416,7 +37416,7 @@
       </c>
       <c r="C1000" s="2" t="inlineStr">
         <is>
-          <t>FOPX</t>
+          <t>FOPX-614</t>
         </is>
       </c>
       <c r="D1000" s="2" t="inlineStr"/>
@@ -37451,7 +37451,7 @@
       </c>
       <c r="C1001" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-705</t>
         </is>
       </c>
       <c r="D1001" s="4" t="inlineStr"/>
@@ -37486,7 +37486,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-705</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr"/>
@@ -37521,7 +37521,7 @@
       </c>
       <c r="C1003" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-705</t>
         </is>
       </c>
       <c r="D1003" s="4" t="inlineStr"/>
@@ -37556,7 +37556,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-705</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr"/>
@@ -37591,7 +37591,7 @@
       </c>
       <c r="C1005" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-705</t>
         </is>
       </c>
       <c r="D1005" s="4" t="inlineStr"/>
@@ -37626,7 +37626,7 @@
       </c>
       <c r="C1006" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-707</t>
         </is>
       </c>
       <c r="D1006" s="2" t="inlineStr"/>
@@ -37661,7 +37661,7 @@
       </c>
       <c r="C1007" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-707</t>
         </is>
       </c>
       <c r="D1007" s="4" t="inlineStr"/>
@@ -37696,7 +37696,7 @@
       </c>
       <c r="C1008" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-707</t>
         </is>
       </c>
       <c r="D1008" s="2" t="inlineStr"/>
@@ -37731,7 +37731,7 @@
       </c>
       <c r="C1009" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-707</t>
         </is>
       </c>
       <c r="D1009" s="4" t="inlineStr"/>
@@ -37766,7 +37766,7 @@
       </c>
       <c r="C1010" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-707</t>
         </is>
       </c>
       <c r="D1010" s="2" t="inlineStr"/>
@@ -37801,7 +37801,7 @@
       </c>
       <c r="C1011" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-709</t>
         </is>
       </c>
       <c r="D1011" s="4" t="inlineStr"/>
@@ -37836,7 +37836,7 @@
       </c>
       <c r="C1012" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-709</t>
         </is>
       </c>
       <c r="D1012" s="2" t="inlineStr"/>
@@ -37871,7 +37871,7 @@
       </c>
       <c r="C1013" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-709</t>
         </is>
       </c>
       <c r="D1013" s="4" t="inlineStr"/>
@@ -37906,7 +37906,7 @@
       </c>
       <c r="C1014" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-709</t>
         </is>
       </c>
       <c r="D1014" s="2" t="inlineStr"/>
@@ -37941,7 +37941,7 @@
       </c>
       <c r="C1015" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-709</t>
         </is>
       </c>
       <c r="D1015" s="4" t="inlineStr"/>
@@ -37976,7 +37976,7 @@
       </c>
       <c r="C1016" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-710</t>
         </is>
       </c>
       <c r="D1016" s="2" t="inlineStr"/>
@@ -38011,7 +38011,7 @@
       </c>
       <c r="C1017" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-710</t>
         </is>
       </c>
       <c r="D1017" s="4" t="inlineStr"/>
@@ -38046,7 +38046,7 @@
       </c>
       <c r="C1018" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-710</t>
         </is>
       </c>
       <c r="D1018" s="2" t="inlineStr"/>
@@ -38081,7 +38081,7 @@
       </c>
       <c r="C1019" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-710</t>
         </is>
       </c>
       <c r="D1019" s="4" t="inlineStr"/>
@@ -38116,7 +38116,7 @@
       </c>
       <c r="C1020" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-710</t>
         </is>
       </c>
       <c r="D1020" s="2" t="inlineStr"/>
@@ -38151,7 +38151,7 @@
       </c>
       <c r="C1021" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-711</t>
         </is>
       </c>
       <c r="D1021" s="4" t="inlineStr"/>
@@ -38186,7 +38186,7 @@
       </c>
       <c r="C1022" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-711</t>
         </is>
       </c>
       <c r="D1022" s="2" t="inlineStr"/>
@@ -38221,7 +38221,7 @@
       </c>
       <c r="C1023" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-711</t>
         </is>
       </c>
       <c r="D1023" s="4" t="inlineStr"/>
@@ -38256,7 +38256,7 @@
       </c>
       <c r="C1024" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-711</t>
         </is>
       </c>
       <c r="D1024" s="2" t="inlineStr"/>
@@ -38291,7 +38291,7 @@
       </c>
       <c r="C1025" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-711</t>
         </is>
       </c>
       <c r="D1025" s="4" t="inlineStr"/>
@@ -38326,7 +38326,7 @@
       </c>
       <c r="C1026" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-713</t>
         </is>
       </c>
       <c r="D1026" s="2" t="inlineStr"/>
@@ -38361,7 +38361,7 @@
       </c>
       <c r="C1027" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-713</t>
         </is>
       </c>
       <c r="D1027" s="4" t="inlineStr"/>
@@ -38396,7 +38396,7 @@
       </c>
       <c r="C1028" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-713</t>
         </is>
       </c>
       <c r="D1028" s="2" t="inlineStr"/>
@@ -38431,7 +38431,7 @@
       </c>
       <c r="C1029" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-713</t>
         </is>
       </c>
       <c r="D1029" s="4" t="inlineStr"/>
@@ -38466,7 +38466,7 @@
       </c>
       <c r="C1030" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-713</t>
         </is>
       </c>
       <c r="D1030" s="2" t="inlineStr"/>
@@ -38501,7 +38501,7 @@
       </c>
       <c r="C1031" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-714</t>
         </is>
       </c>
       <c r="D1031" s="4" t="inlineStr"/>
@@ -38536,7 +38536,7 @@
       </c>
       <c r="C1032" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-714</t>
         </is>
       </c>
       <c r="D1032" s="2" t="inlineStr"/>
@@ -38571,7 +38571,7 @@
       </c>
       <c r="C1033" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-714</t>
         </is>
       </c>
       <c r="D1033" s="4" t="inlineStr"/>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="C1034" s="2" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-714</t>
         </is>
       </c>
       <c r="D1034" s="2" t="inlineStr"/>
@@ -38641,7 +38641,7 @@
       </c>
       <c r="C1035" s="4" t="inlineStr">
         <is>
-          <t>LOPX</t>
+          <t>LOPX-714</t>
         </is>
       </c>
       <c r="D1035" s="4" t="inlineStr"/>
@@ -38676,7 +38676,7 @@
       </c>
       <c r="C1036" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-102</t>
         </is>
       </c>
       <c r="D1036" s="2" t="inlineStr"/>
@@ -38711,7 +38711,7 @@
       </c>
       <c r="C1037" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-102</t>
         </is>
       </c>
       <c r="D1037" s="4" t="inlineStr"/>
@@ -38746,7 +38746,7 @@
       </c>
       <c r="C1038" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-102</t>
         </is>
       </c>
       <c r="D1038" s="2" t="inlineStr"/>
@@ -38781,7 +38781,7 @@
       </c>
       <c r="C1039" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-102</t>
         </is>
       </c>
       <c r="D1039" s="4" t="inlineStr"/>
@@ -38816,7 +38816,7 @@
       </c>
       <c r="C1040" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-102</t>
         </is>
       </c>
       <c r="D1040" s="2" t="inlineStr"/>
@@ -38851,7 +38851,7 @@
       </c>
       <c r="C1041" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-103</t>
         </is>
       </c>
       <c r="D1041" s="4" t="inlineStr"/>
@@ -38886,7 +38886,7 @@
       </c>
       <c r="C1042" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-103</t>
         </is>
       </c>
       <c r="D1042" s="2" t="inlineStr"/>
@@ -38921,7 +38921,7 @@
       </c>
       <c r="C1043" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-103</t>
         </is>
       </c>
       <c r="D1043" s="4" t="inlineStr"/>
@@ -38956,7 +38956,7 @@
       </c>
       <c r="C1044" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-103</t>
         </is>
       </c>
       <c r="D1044" s="2" t="inlineStr"/>
@@ -38991,7 +38991,7 @@
       </c>
       <c r="C1045" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-103</t>
         </is>
       </c>
       <c r="D1045" s="4" t="inlineStr"/>
@@ -39026,7 +39026,7 @@
       </c>
       <c r="C1046" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-104</t>
         </is>
       </c>
       <c r="D1046" s="2" t="inlineStr"/>
@@ -39061,7 +39061,7 @@
       </c>
       <c r="C1047" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-104</t>
         </is>
       </c>
       <c r="D1047" s="4" t="inlineStr"/>
@@ -39096,7 +39096,7 @@
       </c>
       <c r="C1048" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-104</t>
         </is>
       </c>
       <c r="D1048" s="2" t="inlineStr"/>
@@ -39131,7 +39131,7 @@
       </c>
       <c r="C1049" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-104</t>
         </is>
       </c>
       <c r="D1049" s="4" t="inlineStr"/>
@@ -39166,7 +39166,7 @@
       </c>
       <c r="C1050" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-104</t>
         </is>
       </c>
       <c r="D1050" s="2" t="inlineStr"/>
@@ -39201,7 +39201,7 @@
       </c>
       <c r="C1051" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-204</t>
         </is>
       </c>
       <c r="D1051" s="4" t="inlineStr"/>
@@ -39236,7 +39236,7 @@
       </c>
       <c r="C1052" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-204</t>
         </is>
       </c>
       <c r="D1052" s="2" t="inlineStr"/>
@@ -39271,7 +39271,7 @@
       </c>
       <c r="C1053" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-204</t>
         </is>
       </c>
       <c r="D1053" s="4" t="inlineStr"/>
@@ -39306,7 +39306,7 @@
       </c>
       <c r="C1054" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-204</t>
         </is>
       </c>
       <c r="D1054" s="2" t="inlineStr"/>
@@ -39341,7 +39341,7 @@
       </c>
       <c r="C1055" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-204</t>
         </is>
       </c>
       <c r="D1055" s="4" t="inlineStr"/>
@@ -39376,7 +39376,7 @@
       </c>
       <c r="C1056" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-205</t>
         </is>
       </c>
       <c r="D1056" s="2" t="inlineStr"/>
@@ -39411,7 +39411,7 @@
       </c>
       <c r="C1057" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-205</t>
         </is>
       </c>
       <c r="D1057" s="4" t="inlineStr"/>
@@ -39446,7 +39446,7 @@
       </c>
       <c r="C1058" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-205</t>
         </is>
       </c>
       <c r="D1058" s="2" t="inlineStr"/>
@@ -39481,7 +39481,7 @@
       </c>
       <c r="C1059" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-205</t>
         </is>
       </c>
       <c r="D1059" s="4" t="inlineStr"/>
@@ -39516,7 +39516,7 @@
       </c>
       <c r="C1060" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-205</t>
         </is>
       </c>
       <c r="D1060" s="2" t="inlineStr"/>
@@ -39551,7 +39551,7 @@
       </c>
       <c r="C1061" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-206</t>
         </is>
       </c>
       <c r="D1061" s="4" t="inlineStr"/>
@@ -39586,7 +39586,7 @@
       </c>
       <c r="C1062" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-206</t>
         </is>
       </c>
       <c r="D1062" s="2" t="inlineStr"/>
@@ -39621,7 +39621,7 @@
       </c>
       <c r="C1063" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-206</t>
         </is>
       </c>
       <c r="D1063" s="4" t="inlineStr"/>
@@ -39656,7 +39656,7 @@
       </c>
       <c r="C1064" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-206</t>
         </is>
       </c>
       <c r="D1064" s="2" t="inlineStr"/>
@@ -39691,7 +39691,7 @@
       </c>
       <c r="C1065" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-206</t>
         </is>
       </c>
       <c r="D1065" s="4" t="inlineStr"/>
@@ -39726,7 +39726,7 @@
       </c>
       <c r="C1066" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-207</t>
         </is>
       </c>
       <c r="D1066" s="2" t="inlineStr"/>
@@ -39761,7 +39761,7 @@
       </c>
       <c r="C1067" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-207</t>
         </is>
       </c>
       <c r="D1067" s="4" t="inlineStr"/>
@@ -39796,7 +39796,7 @@
       </c>
       <c r="C1068" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-207</t>
         </is>
       </c>
       <c r="D1068" s="2" t="inlineStr"/>
@@ -39831,7 +39831,7 @@
       </c>
       <c r="C1069" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-207</t>
         </is>
       </c>
       <c r="D1069" s="4" t="inlineStr"/>
@@ -39866,7 +39866,7 @@
       </c>
       <c r="C1070" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-207</t>
         </is>
       </c>
       <c r="D1070" s="2" t="inlineStr"/>
@@ -39901,7 +39901,7 @@
       </c>
       <c r="C1071" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-209</t>
         </is>
       </c>
       <c r="D1071" s="4" t="inlineStr"/>
@@ -39936,7 +39936,7 @@
       </c>
       <c r="C1072" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-209</t>
         </is>
       </c>
       <c r="D1072" s="2" t="inlineStr"/>
@@ -39971,7 +39971,7 @@
       </c>
       <c r="C1073" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-209</t>
         </is>
       </c>
       <c r="D1073" s="4" t="inlineStr"/>
@@ -40006,7 +40006,7 @@
       </c>
       <c r="C1074" s="2" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-209</t>
         </is>
       </c>
       <c r="D1074" s="2" t="inlineStr"/>
@@ -40041,7 +40041,7 @@
       </c>
       <c r="C1075" s="4" t="inlineStr">
         <is>
-          <t>MAB</t>
+          <t>MAB-209</t>
         </is>
       </c>
       <c r="D1075" s="4" t="inlineStr"/>
@@ -40076,7 +40076,7 @@
       </c>
       <c r="C1076" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-204</t>
         </is>
       </c>
       <c r="D1076" s="2" t="inlineStr"/>
@@ -40111,7 +40111,7 @@
       </c>
       <c r="C1077" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-204</t>
         </is>
       </c>
       <c r="D1077" s="4" t="inlineStr"/>
@@ -40146,7 +40146,7 @@
       </c>
       <c r="C1078" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-204</t>
         </is>
       </c>
       <c r="D1078" s="2" t="inlineStr"/>
@@ -40181,7 +40181,7 @@
       </c>
       <c r="C1079" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-204</t>
         </is>
       </c>
       <c r="D1079" s="4" t="inlineStr"/>
@@ -40216,7 +40216,7 @@
       </c>
       <c r="C1080" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-204</t>
         </is>
       </c>
       <c r="D1080" s="2" t="inlineStr"/>
@@ -40251,7 +40251,7 @@
       </c>
       <c r="C1081" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-205</t>
         </is>
       </c>
       <c r="D1081" s="4" t="inlineStr"/>
@@ -40286,7 +40286,7 @@
       </c>
       <c r="C1082" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-205</t>
         </is>
       </c>
       <c r="D1082" s="2" t="inlineStr"/>
@@ -40321,7 +40321,7 @@
       </c>
       <c r="C1083" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-205</t>
         </is>
       </c>
       <c r="D1083" s="4" t="inlineStr"/>
@@ -40356,7 +40356,7 @@
       </c>
       <c r="C1084" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-205</t>
         </is>
       </c>
       <c r="D1084" s="2" t="inlineStr"/>
@@ -40391,7 +40391,7 @@
       </c>
       <c r="C1085" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-205</t>
         </is>
       </c>
       <c r="D1085" s="4" t="inlineStr"/>
@@ -40426,7 +40426,7 @@
       </c>
       <c r="C1086" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-207</t>
         </is>
       </c>
       <c r="D1086" s="2" t="inlineStr"/>
@@ -40461,7 +40461,7 @@
       </c>
       <c r="C1087" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-207</t>
         </is>
       </c>
       <c r="D1087" s="4" t="inlineStr"/>
@@ -40496,7 +40496,7 @@
       </c>
       <c r="C1088" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-207</t>
         </is>
       </c>
       <c r="D1088" s="2" t="inlineStr"/>
@@ -40531,7 +40531,7 @@
       </c>
       <c r="C1089" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-210</t>
         </is>
       </c>
       <c r="D1089" s="4" t="inlineStr"/>
@@ -40566,7 +40566,7 @@
       </c>
       <c r="C1090" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-210</t>
         </is>
       </c>
       <c r="D1090" s="2" t="inlineStr"/>
@@ -40601,7 +40601,7 @@
       </c>
       <c r="C1091" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-210</t>
         </is>
       </c>
       <c r="D1091" s="4" t="inlineStr"/>
@@ -40636,7 +40636,7 @@
       </c>
       <c r="C1092" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-210</t>
         </is>
       </c>
       <c r="D1092" s="2" t="inlineStr"/>
@@ -40671,7 +40671,7 @@
       </c>
       <c r="C1093" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-210</t>
         </is>
       </c>
       <c r="D1093" s="4" t="inlineStr"/>
@@ -40706,7 +40706,7 @@
       </c>
       <c r="C1094" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-309</t>
         </is>
       </c>
       <c r="D1094" s="2" t="inlineStr"/>
@@ -40741,7 +40741,7 @@
       </c>
       <c r="C1095" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-309</t>
         </is>
       </c>
       <c r="D1095" s="4" t="inlineStr"/>
@@ -40776,7 +40776,7 @@
       </c>
       <c r="C1096" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-309</t>
         </is>
       </c>
       <c r="D1096" s="2" t="inlineStr"/>
@@ -40811,7 +40811,7 @@
       </c>
       <c r="C1097" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-309</t>
         </is>
       </c>
       <c r="D1097" s="4" t="inlineStr"/>
@@ -40846,7 +40846,7 @@
       </c>
       <c r="C1098" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-309</t>
         </is>
       </c>
       <c r="D1098" s="2" t="inlineStr"/>
@@ -40881,7 +40881,7 @@
       </c>
       <c r="C1099" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-313</t>
         </is>
       </c>
       <c r="D1099" s="4" t="inlineStr"/>
@@ -40916,7 +40916,7 @@
       </c>
       <c r="C1100" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-313</t>
         </is>
       </c>
       <c r="D1100" s="2" t="inlineStr"/>
@@ -40951,7 +40951,7 @@
       </c>
       <c r="C1101" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-313</t>
         </is>
       </c>
       <c r="D1101" s="4" t="inlineStr"/>
@@ -40986,7 +40986,7 @@
       </c>
       <c r="C1102" s="2" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-313</t>
         </is>
       </c>
       <c r="D1102" s="2" t="inlineStr"/>
@@ -41021,7 +41021,7 @@
       </c>
       <c r="C1103" s="4" t="inlineStr">
         <is>
-          <t>MAPX</t>
+          <t>MAPX-313</t>
         </is>
       </c>
       <c r="D1103" s="4" t="inlineStr"/>
@@ -41056,7 +41056,7 @@
       </c>
       <c r="C1104" s="2" t="inlineStr">
         <is>
-          <t>MFPX</t>
+          <t>MFPX-307</t>
         </is>
       </c>
       <c r="D1104" s="2" t="inlineStr"/>
@@ -41091,7 +41091,7 @@
       </c>
       <c r="C1105" s="4" t="inlineStr">
         <is>
-          <t>MFPX</t>
+          <t>MFPX-307</t>
         </is>
       </c>
       <c r="D1105" s="4" t="inlineStr"/>
@@ -41126,7 +41126,7 @@
       </c>
       <c r="C1106" s="2" t="inlineStr">
         <is>
-          <t>MFPX</t>
+          <t>MFPX-307</t>
         </is>
       </c>
       <c r="D1106" s="2" t="inlineStr"/>
@@ -41161,7 +41161,7 @@
       </c>
       <c r="C1107" s="4" t="inlineStr">
         <is>
-          <t>MFPX</t>
+          <t>MFPX-307</t>
         </is>
       </c>
       <c r="D1107" s="4" t="inlineStr"/>
@@ -41196,7 +41196,7 @@
       </c>
       <c r="C1108" s="2" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-304</t>
         </is>
       </c>
       <c r="D1108" s="2" t="inlineStr"/>
@@ -41231,7 +41231,7 @@
       </c>
       <c r="C1109" s="4" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-304</t>
         </is>
       </c>
       <c r="D1109" s="4" t="inlineStr"/>
@@ -41266,7 +41266,7 @@
       </c>
       <c r="C1110" s="2" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-304</t>
         </is>
       </c>
       <c r="D1110" s="2" t="inlineStr"/>
@@ -41301,7 +41301,7 @@
       </c>
       <c r="C1111" s="4" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-304</t>
         </is>
       </c>
       <c r="D1111" s="4" t="inlineStr"/>
@@ -41336,7 +41336,7 @@
       </c>
       <c r="C1112" s="2" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-305</t>
         </is>
       </c>
       <c r="D1112" s="2" t="inlineStr"/>
@@ -41371,7 +41371,7 @@
       </c>
       <c r="C1113" s="4" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-305</t>
         </is>
       </c>
       <c r="D1113" s="4" t="inlineStr"/>
@@ -41406,7 +41406,7 @@
       </c>
       <c r="C1114" s="2" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-305</t>
         </is>
       </c>
       <c r="D1114" s="2" t="inlineStr"/>
@@ -41441,7 +41441,7 @@
       </c>
       <c r="C1115" s="4" t="inlineStr">
         <is>
-          <t>MMB</t>
+          <t>MMB-305</t>
         </is>
       </c>
       <c r="D1115" s="4" t="inlineStr"/>
@@ -41476,7 +41476,7 @@
       </c>
       <c r="C1116" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-303</t>
         </is>
       </c>
       <c r="D1116" s="2" t="inlineStr"/>
@@ -41511,7 +41511,7 @@
       </c>
       <c r="C1117" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-303</t>
         </is>
       </c>
       <c r="D1117" s="4" t="inlineStr"/>
@@ -41546,7 +41546,7 @@
       </c>
       <c r="C1118" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-303</t>
         </is>
       </c>
       <c r="D1118" s="2" t="inlineStr"/>
@@ -41581,7 +41581,7 @@
       </c>
       <c r="C1119" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-303</t>
         </is>
       </c>
       <c r="D1119" s="4" t="inlineStr"/>
@@ -41616,7 +41616,7 @@
       </c>
       <c r="C1120" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-304</t>
         </is>
       </c>
       <c r="D1120" s="2" t="inlineStr"/>
@@ -41651,7 +41651,7 @@
       </c>
       <c r="C1121" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-304</t>
         </is>
       </c>
       <c r="D1121" s="4" t="inlineStr"/>
@@ -41686,7 +41686,7 @@
       </c>
       <c r="C1122" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-304</t>
         </is>
       </c>
       <c r="D1122" s="2" t="inlineStr"/>
@@ -41721,7 +41721,7 @@
       </c>
       <c r="C1123" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-304</t>
         </is>
       </c>
       <c r="D1123" s="4" t="inlineStr"/>
@@ -41756,7 +41756,7 @@
       </c>
       <c r="C1124" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-403</t>
         </is>
       </c>
       <c r="D1124" s="2" t="inlineStr"/>
@@ -41791,7 +41791,7 @@
       </c>
       <c r="C1125" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-403</t>
         </is>
       </c>
       <c r="D1125" s="4" t="inlineStr"/>
@@ -41826,7 +41826,7 @@
       </c>
       <c r="C1126" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-403</t>
         </is>
       </c>
       <c r="D1126" s="2" t="inlineStr"/>
@@ -41861,7 +41861,7 @@
       </c>
       <c r="C1127" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-403</t>
         </is>
       </c>
       <c r="D1127" s="4" t="inlineStr"/>
@@ -41896,7 +41896,7 @@
       </c>
       <c r="C1128" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-404</t>
         </is>
       </c>
       <c r="D1128" s="2" t="inlineStr"/>
@@ -41931,7 +41931,7 @@
       </c>
       <c r="C1129" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-404</t>
         </is>
       </c>
       <c r="D1129" s="4" t="inlineStr"/>
@@ -41966,7 +41966,7 @@
       </c>
       <c r="C1130" s="2" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-404</t>
         </is>
       </c>
       <c r="D1130" s="2" t="inlineStr"/>
@@ -42001,7 +42001,7 @@
       </c>
       <c r="C1131" s="4" t="inlineStr">
         <is>
-          <t>MMPX</t>
+          <t>MMPX-404</t>
         </is>
       </c>
       <c r="D1131" s="4" t="inlineStr"/>
@@ -42036,7 +42036,7 @@
       </c>
       <c r="C1132" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-204</t>
         </is>
       </c>
       <c r="D1132" s="2" t="inlineStr"/>
@@ -42071,7 +42071,7 @@
       </c>
       <c r="C1133" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-204</t>
         </is>
       </c>
       <c r="D1133" s="4" t="inlineStr"/>
@@ -42106,7 +42106,7 @@
       </c>
       <c r="C1134" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-204</t>
         </is>
       </c>
       <c r="D1134" s="2" t="inlineStr"/>
@@ -42141,7 +42141,7 @@
       </c>
       <c r="C1135" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-204</t>
         </is>
       </c>
       <c r="D1135" s="4" t="inlineStr"/>
@@ -42176,7 +42176,7 @@
       </c>
       <c r="C1136" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-204</t>
         </is>
       </c>
       <c r="D1136" s="2" t="inlineStr"/>
@@ -42211,7 +42211,7 @@
       </c>
       <c r="C1137" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-205</t>
         </is>
       </c>
       <c r="D1137" s="4" t="inlineStr"/>
@@ -42246,7 +42246,7 @@
       </c>
       <c r="C1138" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-205</t>
         </is>
       </c>
       <c r="D1138" s="2" t="inlineStr"/>
@@ -42281,7 +42281,7 @@
       </c>
       <c r="C1139" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-205</t>
         </is>
       </c>
       <c r="D1139" s="4" t="inlineStr"/>
@@ -42316,7 +42316,7 @@
       </c>
       <c r="C1140" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-205</t>
         </is>
       </c>
       <c r="D1140" s="2" t="inlineStr"/>
@@ -42351,7 +42351,7 @@
       </c>
       <c r="C1141" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-205</t>
         </is>
       </c>
       <c r="D1141" s="4" t="inlineStr"/>
@@ -42386,7 +42386,7 @@
       </c>
       <c r="C1142" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-207</t>
         </is>
       </c>
       <c r="D1142" s="2" t="inlineStr"/>
@@ -42421,7 +42421,7 @@
       </c>
       <c r="C1143" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-207</t>
         </is>
       </c>
       <c r="D1143" s="4" t="inlineStr"/>
@@ -42456,7 +42456,7 @@
       </c>
       <c r="C1144" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-207</t>
         </is>
       </c>
       <c r="D1144" s="2" t="inlineStr"/>
@@ -42491,7 +42491,7 @@
       </c>
       <c r="C1145" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-209</t>
         </is>
       </c>
       <c r="D1145" s="4" t="inlineStr"/>
@@ -42526,7 +42526,7 @@
       </c>
       <c r="C1146" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-209</t>
         </is>
       </c>
       <c r="D1146" s="2" t="inlineStr"/>
@@ -42561,7 +42561,7 @@
       </c>
       <c r="C1147" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-209</t>
         </is>
       </c>
       <c r="D1147" s="4" t="inlineStr"/>
@@ -42596,7 +42596,7 @@
       </c>
       <c r="C1148" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-209</t>
         </is>
       </c>
       <c r="D1148" s="2" t="inlineStr"/>
@@ -42631,7 +42631,7 @@
       </c>
       <c r="C1149" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-209</t>
         </is>
       </c>
       <c r="D1149" s="4" t="inlineStr"/>
@@ -42666,7 +42666,7 @@
       </c>
       <c r="C1150" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-210</t>
         </is>
       </c>
       <c r="D1150" s="2" t="inlineStr"/>
@@ -42701,7 +42701,7 @@
       </c>
       <c r="C1151" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-210</t>
         </is>
       </c>
       <c r="D1151" s="4" t="inlineStr"/>
@@ -42736,7 +42736,7 @@
       </c>
       <c r="C1152" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-210</t>
         </is>
       </c>
       <c r="D1152" s="2" t="inlineStr"/>
@@ -42771,7 +42771,7 @@
       </c>
       <c r="C1153" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-210</t>
         </is>
       </c>
       <c r="D1153" s="4" t="inlineStr"/>
@@ -42806,7 +42806,7 @@
       </c>
       <c r="C1154" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-210</t>
         </is>
       </c>
       <c r="D1154" s="2" t="inlineStr"/>
@@ -42841,7 +42841,7 @@
       </c>
       <c r="C1155" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-213</t>
         </is>
       </c>
       <c r="D1155" s="4" t="inlineStr"/>
@@ -42876,7 +42876,7 @@
       </c>
       <c r="C1156" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-213</t>
         </is>
       </c>
       <c r="D1156" s="2" t="inlineStr"/>
@@ -42911,7 +42911,7 @@
       </c>
       <c r="C1157" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-213</t>
         </is>
       </c>
       <c r="D1157" s="4" t="inlineStr"/>
@@ -42946,7 +42946,7 @@
       </c>
       <c r="C1158" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-213</t>
         </is>
       </c>
       <c r="D1158" s="2" t="inlineStr"/>
@@ -42981,7 +42981,7 @@
       </c>
       <c r="C1159" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-213</t>
         </is>
       </c>
       <c r="D1159" s="4" t="inlineStr"/>
@@ -43016,7 +43016,7 @@
       </c>
       <c r="C1160" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-309</t>
         </is>
       </c>
       <c r="D1160" s="2" t="inlineStr"/>
@@ -43051,7 +43051,7 @@
       </c>
       <c r="C1161" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-309</t>
         </is>
       </c>
       <c r="D1161" s="4" t="inlineStr"/>
@@ -43086,7 +43086,7 @@
       </c>
       <c r="C1162" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-309</t>
         </is>
       </c>
       <c r="D1162" s="2" t="inlineStr"/>
@@ -43121,7 +43121,7 @@
       </c>
       <c r="C1163" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-309</t>
         </is>
       </c>
       <c r="D1163" s="4" t="inlineStr"/>
@@ -43156,7 +43156,7 @@
       </c>
       <c r="C1164" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-309</t>
         </is>
       </c>
       <c r="D1164" s="2" t="inlineStr"/>
@@ -43191,7 +43191,7 @@
       </c>
       <c r="C1165" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-310</t>
         </is>
       </c>
       <c r="D1165" s="4" t="inlineStr"/>
@@ -43226,7 +43226,7 @@
       </c>
       <c r="C1166" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-310</t>
         </is>
       </c>
       <c r="D1166" s="2" t="inlineStr"/>
@@ -43261,7 +43261,7 @@
       </c>
       <c r="C1167" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-310</t>
         </is>
       </c>
       <c r="D1167" s="4" t="inlineStr"/>
@@ -43296,7 +43296,7 @@
       </c>
       <c r="C1168" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-310</t>
         </is>
       </c>
       <c r="D1168" s="2" t="inlineStr"/>
@@ -43331,7 +43331,7 @@
       </c>
       <c r="C1169" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-310</t>
         </is>
       </c>
       <c r="D1169" s="4" t="inlineStr"/>
@@ -43366,7 +43366,7 @@
       </c>
       <c r="C1170" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-313</t>
         </is>
       </c>
       <c r="D1170" s="2" t="inlineStr"/>
@@ -43401,7 +43401,7 @@
       </c>
       <c r="C1171" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-313</t>
         </is>
       </c>
       <c r="D1171" s="4" t="inlineStr"/>
@@ -43436,7 +43436,7 @@
       </c>
       <c r="C1172" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-313</t>
         </is>
       </c>
       <c r="D1172" s="2" t="inlineStr"/>
@@ -43471,7 +43471,7 @@
       </c>
       <c r="C1173" s="4" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-313</t>
         </is>
       </c>
       <c r="D1173" s="4" t="inlineStr"/>
@@ -43506,7 +43506,7 @@
       </c>
       <c r="C1174" s="2" t="inlineStr">
         <is>
-          <t>MOPX</t>
+          <t>MOPX-313</t>
         </is>
       </c>
       <c r="D1174" s="2" t="inlineStr"/>
@@ -43541,7 +43541,7 @@
       </c>
       <c r="C1175" s="4" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-303</t>
         </is>
       </c>
       <c r="D1175" s="4" t="inlineStr"/>
@@ -43576,7 +43576,7 @@
       </c>
       <c r="C1176" s="2" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-303</t>
         </is>
       </c>
       <c r="D1176" s="2" t="inlineStr"/>
@@ -43611,7 +43611,7 @@
       </c>
       <c r="C1177" s="4" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-303</t>
         </is>
       </c>
       <c r="D1177" s="4" t="inlineStr"/>
@@ -43646,7 +43646,7 @@
       </c>
       <c r="C1178" s="2" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-303</t>
         </is>
       </c>
       <c r="D1178" s="2" t="inlineStr"/>
@@ -43681,7 +43681,7 @@
       </c>
       <c r="C1179" s="4" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-403</t>
         </is>
       </c>
       <c r="D1179" s="4" t="inlineStr"/>
@@ -43716,7 +43716,7 @@
       </c>
       <c r="C1180" s="2" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-403</t>
         </is>
       </c>
       <c r="D1180" s="2" t="inlineStr"/>
@@ -43751,7 +43751,7 @@
       </c>
       <c r="C1181" s="4" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-403</t>
         </is>
       </c>
       <c r="D1181" s="4" t="inlineStr"/>
@@ -43786,7 +43786,7 @@
       </c>
       <c r="C1182" s="2" t="inlineStr">
         <is>
-          <t>MSPX</t>
+          <t>MSPX-403</t>
         </is>
       </c>
       <c r="D1182" s="2" t="inlineStr"/>
@@ -43821,7 +43821,7 @@
       </c>
       <c r="C1183" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-600</t>
         </is>
       </c>
       <c r="D1183" s="4" t="inlineStr"/>
@@ -43856,7 +43856,7 @@
       </c>
       <c r="C1184" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-600</t>
         </is>
       </c>
       <c r="D1184" s="2" t="inlineStr"/>
@@ -43891,7 +43891,7 @@
       </c>
       <c r="C1185" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-600</t>
         </is>
       </c>
       <c r="D1185" s="4" t="inlineStr"/>
@@ -43926,7 +43926,7 @@
       </c>
       <c r="C1186" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-600</t>
         </is>
       </c>
       <c r="D1186" s="2" t="inlineStr"/>
@@ -43961,7 +43961,7 @@
       </c>
       <c r="C1187" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-605</t>
         </is>
       </c>
       <c r="D1187" s="4" t="inlineStr"/>
@@ -43996,7 +43996,7 @@
       </c>
       <c r="C1188" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-605</t>
         </is>
       </c>
       <c r="D1188" s="2" t="inlineStr"/>
@@ -44031,7 +44031,7 @@
       </c>
       <c r="C1189" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-605</t>
         </is>
       </c>
       <c r="D1189" s="4" t="inlineStr"/>
@@ -44066,7 +44066,7 @@
       </c>
       <c r="C1190" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-605</t>
         </is>
       </c>
       <c r="D1190" s="2" t="inlineStr"/>
@@ -44101,7 +44101,7 @@
       </c>
       <c r="C1191" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-610</t>
         </is>
       </c>
       <c r="D1191" s="4" t="inlineStr"/>
@@ -44136,7 +44136,7 @@
       </c>
       <c r="C1192" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-610</t>
         </is>
       </c>
       <c r="D1192" s="2" t="inlineStr"/>
@@ -44171,7 +44171,7 @@
       </c>
       <c r="C1193" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-610</t>
         </is>
       </c>
       <c r="D1193" s="4" t="inlineStr"/>
@@ -44206,7 +44206,7 @@
       </c>
       <c r="C1194" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-610</t>
         </is>
       </c>
       <c r="D1194" s="2" t="inlineStr"/>
@@ -44241,7 +44241,7 @@
       </c>
       <c r="C1195" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-615</t>
         </is>
       </c>
       <c r="D1195" s="4" t="inlineStr"/>
@@ -44276,7 +44276,7 @@
       </c>
       <c r="C1196" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-615</t>
         </is>
       </c>
       <c r="D1196" s="2" t="inlineStr"/>
@@ -44311,7 +44311,7 @@
       </c>
       <c r="C1197" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-615</t>
         </is>
       </c>
       <c r="D1197" s="4" t="inlineStr"/>
@@ -44346,7 +44346,7 @@
       </c>
       <c r="C1198" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-615</t>
         </is>
       </c>
       <c r="D1198" s="2" t="inlineStr"/>
@@ -44381,7 +44381,7 @@
       </c>
       <c r="C1199" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-625</t>
         </is>
       </c>
       <c r="D1199" s="4" t="inlineStr">
@@ -44420,7 +44420,7 @@
       </c>
       <c r="C1200" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-625</t>
         </is>
       </c>
       <c r="D1200" s="2" t="inlineStr">
@@ -44459,7 +44459,7 @@
       </c>
       <c r="C1201" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-635</t>
         </is>
       </c>
       <c r="D1201" s="4" t="inlineStr">
@@ -44498,7 +44498,7 @@
       </c>
       <c r="C1202" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA-635</t>
         </is>
       </c>
       <c r="D1202" s="2" t="inlineStr">
@@ -44537,7 +44537,7 @@
       </c>
       <c r="C1203" s="4" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-100</t>
         </is>
       </c>
       <c r="D1203" s="4" t="inlineStr"/>
@@ -44572,7 +44572,7 @@
       </c>
       <c r="C1204" s="2" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-100</t>
         </is>
       </c>
       <c r="D1204" s="2" t="inlineStr"/>
@@ -44607,7 +44607,7 @@
       </c>
       <c r="C1205" s="4" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-100</t>
         </is>
       </c>
       <c r="D1205" s="4" t="inlineStr"/>
@@ -44642,7 +44642,7 @@
       </c>
       <c r="C1206" s="2" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-100</t>
         </is>
       </c>
       <c r="D1206" s="2" t="inlineStr"/>
@@ -44677,7 +44677,7 @@
       </c>
       <c r="C1207" s="4" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-150</t>
         </is>
       </c>
       <c r="D1207" s="4" t="inlineStr"/>
@@ -44712,7 +44712,7 @@
       </c>
       <c r="C1208" s="2" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-150</t>
         </is>
       </c>
       <c r="D1208" s="2" t="inlineStr"/>
@@ -44747,7 +44747,7 @@
       </c>
       <c r="C1209" s="4" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-150</t>
         </is>
       </c>
       <c r="D1209" s="4" t="inlineStr"/>
@@ -44782,7 +44782,7 @@
       </c>
       <c r="C1210" s="2" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>PU-150</t>
         </is>
       </c>
       <c r="D1210" s="2" t="inlineStr"/>
@@ -44817,7 +44817,7 @@
       </c>
       <c r="C1211" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-300</t>
         </is>
       </c>
       <c r="D1211" s="4" t="inlineStr">
@@ -44856,7 +44856,7 @@
       </c>
       <c r="C1212" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-300</t>
         </is>
       </c>
       <c r="D1212" s="2" t="inlineStr">
@@ -44895,7 +44895,7 @@
       </c>
       <c r="C1213" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-300</t>
         </is>
       </c>
       <c r="D1213" s="4" t="inlineStr">
@@ -44934,7 +44934,7 @@
       </c>
       <c r="C1214" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-500</t>
         </is>
       </c>
       <c r="D1214" s="2" t="inlineStr">
@@ -44973,7 +44973,7 @@
       </c>
       <c r="C1215" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-500</t>
         </is>
       </c>
       <c r="D1215" s="4" t="inlineStr">
@@ -45012,7 +45012,7 @@
       </c>
       <c r="C1216" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-500</t>
         </is>
       </c>
       <c r="D1216" s="2" t="inlineStr">
@@ -45051,7 +45051,7 @@
       </c>
       <c r="C1217" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-811</t>
         </is>
       </c>
       <c r="D1217" s="4" t="inlineStr">
@@ -45090,7 +45090,7 @@
       </c>
       <c r="C1218" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-811</t>
         </is>
       </c>
       <c r="D1218" s="2" t="inlineStr">
@@ -45129,7 +45129,7 @@
       </c>
       <c r="C1219" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-816</t>
         </is>
       </c>
       <c r="D1219" s="4" t="inlineStr">
@@ -45168,7 +45168,7 @@
       </c>
       <c r="C1220" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-816</t>
         </is>
       </c>
       <c r="D1220" s="2" t="inlineStr">
@@ -45207,7 +45207,7 @@
       </c>
       <c r="C1221" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-820</t>
         </is>
       </c>
       <c r="D1221" s="4" t="inlineStr">
@@ -45246,7 +45246,7 @@
       </c>
       <c r="C1222" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-820</t>
         </is>
       </c>
       <c r="D1222" s="2" t="inlineStr">
@@ -45285,7 +45285,7 @@
       </c>
       <c r="C1223" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-821</t>
         </is>
       </c>
       <c r="D1223" s="4" t="inlineStr">
@@ -45324,7 +45324,7 @@
       </c>
       <c r="C1224" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-821</t>
         </is>
       </c>
       <c r="D1224" s="2" t="inlineStr">
@@ -45363,7 +45363,7 @@
       </c>
       <c r="C1225" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-825</t>
         </is>
       </c>
       <c r="D1225" s="4" t="inlineStr">
@@ -45402,7 +45402,7 @@
       </c>
       <c r="C1226" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-825</t>
         </is>
       </c>
       <c r="D1226" s="2" t="inlineStr">
@@ -45441,7 +45441,7 @@
       </c>
       <c r="C1227" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-826</t>
         </is>
       </c>
       <c r="D1227" s="4" t="inlineStr">
@@ -45480,7 +45480,7 @@
       </c>
       <c r="C1228" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-826</t>
         </is>
       </c>
       <c r="D1228" s="2" t="inlineStr">
@@ -45519,7 +45519,7 @@
       </c>
       <c r="C1229" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-830</t>
         </is>
       </c>
       <c r="D1229" s="4" t="inlineStr">
@@ -45558,7 +45558,7 @@
       </c>
       <c r="C1230" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-830</t>
         </is>
       </c>
       <c r="D1230" s="2" t="inlineStr">
@@ -45597,7 +45597,7 @@
       </c>
       <c r="C1231" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-831</t>
         </is>
       </c>
       <c r="D1231" s="4" t="inlineStr">
@@ -45636,7 +45636,7 @@
       </c>
       <c r="C1232" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-831</t>
         </is>
       </c>
       <c r="D1232" s="2" t="inlineStr">
@@ -45675,7 +45675,7 @@
       </c>
       <c r="C1233" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-835</t>
         </is>
       </c>
       <c r="D1233" s="4" t="inlineStr">
@@ -45714,7 +45714,7 @@
       </c>
       <c r="C1234" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-835</t>
         </is>
       </c>
       <c r="D1234" s="2" t="inlineStr">
@@ -45753,7 +45753,7 @@
       </c>
       <c r="C1235" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-836</t>
         </is>
       </c>
       <c r="D1235" s="4" t="inlineStr">
@@ -45792,7 +45792,7 @@
       </c>
       <c r="C1236" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-836</t>
         </is>
       </c>
       <c r="D1236" s="2" t="inlineStr">
@@ -45831,7 +45831,7 @@
       </c>
       <c r="C1237" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-840</t>
         </is>
       </c>
       <c r="D1237" s="4" t="inlineStr">
@@ -45870,7 +45870,7 @@
       </c>
       <c r="C1238" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-840</t>
         </is>
       </c>
       <c r="D1238" s="2" t="inlineStr">
@@ -45909,7 +45909,7 @@
       </c>
       <c r="C1239" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-841</t>
         </is>
       </c>
       <c r="D1239" s="4" t="inlineStr">
@@ -45948,7 +45948,7 @@
       </c>
       <c r="C1240" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-841</t>
         </is>
       </c>
       <c r="D1240" s="2" t="inlineStr">
@@ -45987,7 +45987,7 @@
       </c>
       <c r="C1241" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-845</t>
         </is>
       </c>
       <c r="D1241" s="4" t="inlineStr">
@@ -46026,7 +46026,7 @@
       </c>
       <c r="C1242" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-845</t>
         </is>
       </c>
       <c r="D1242" s="2" t="inlineStr">
@@ -46065,7 +46065,7 @@
       </c>
       <c r="C1243" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-846</t>
         </is>
       </c>
       <c r="D1243" s="4" t="inlineStr">
@@ -46104,7 +46104,7 @@
       </c>
       <c r="C1244" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-846</t>
         </is>
       </c>
       <c r="D1244" s="2" t="inlineStr">
@@ -46143,7 +46143,7 @@
       </c>
       <c r="C1245" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-850</t>
         </is>
       </c>
       <c r="D1245" s="4" t="inlineStr">
@@ -46182,7 +46182,7 @@
       </c>
       <c r="C1246" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-850</t>
         </is>
       </c>
       <c r="D1246" s="2" t="inlineStr">
@@ -46221,7 +46221,7 @@
       </c>
       <c r="C1247" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-851</t>
         </is>
       </c>
       <c r="D1247" s="4" t="inlineStr">
@@ -46260,7 +46260,7 @@
       </c>
       <c r="C1248" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-851</t>
         </is>
       </c>
       <c r="D1248" s="2" t="inlineStr">
@@ -46299,7 +46299,7 @@
       </c>
       <c r="C1249" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-855</t>
         </is>
       </c>
       <c r="D1249" s="4" t="inlineStr">
@@ -46338,7 +46338,7 @@
       </c>
       <c r="C1250" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-855</t>
         </is>
       </c>
       <c r="D1250" s="2" t="inlineStr">
@@ -46377,7 +46377,7 @@
       </c>
       <c r="C1251" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-856</t>
         </is>
       </c>
       <c r="D1251" s="4" t="inlineStr">
@@ -46416,7 +46416,7 @@
       </c>
       <c r="C1252" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-856</t>
         </is>
       </c>
       <c r="D1252" s="2" t="inlineStr">
@@ -46455,7 +46455,7 @@
       </c>
       <c r="C1253" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-860</t>
         </is>
       </c>
       <c r="D1253" s="4" t="inlineStr">
@@ -46494,7 +46494,7 @@
       </c>
       <c r="C1254" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-860</t>
         </is>
       </c>
       <c r="D1254" s="2" t="inlineStr">
@@ -46533,7 +46533,7 @@
       </c>
       <c r="C1255" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-861</t>
         </is>
       </c>
       <c r="D1255" s="4" t="inlineStr">
@@ -46572,7 +46572,7 @@
       </c>
       <c r="C1256" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-861</t>
         </is>
       </c>
       <c r="D1256" s="2" t="inlineStr">
@@ -46611,7 +46611,7 @@
       </c>
       <c r="C1257" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-865</t>
         </is>
       </c>
       <c r="D1257" s="4" t="inlineStr">
@@ -46650,7 +46650,7 @@
       </c>
       <c r="C1258" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-865</t>
         </is>
       </c>
       <c r="D1258" s="2" t="inlineStr">
@@ -46689,7 +46689,7 @@
       </c>
       <c r="C1259" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-866</t>
         </is>
       </c>
       <c r="D1259" s="4" t="inlineStr">
@@ -46728,7 +46728,7 @@
       </c>
       <c r="C1260" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-866</t>
         </is>
       </c>
       <c r="D1260" s="2" t="inlineStr">
@@ -46767,7 +46767,7 @@
       </c>
       <c r="C1261" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-870</t>
         </is>
       </c>
       <c r="D1261" s="4" t="inlineStr">
@@ -46806,7 +46806,7 @@
       </c>
       <c r="C1262" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-870</t>
         </is>
       </c>
       <c r="D1262" s="2" t="inlineStr">
@@ -46845,7 +46845,7 @@
       </c>
       <c r="C1263" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-871</t>
         </is>
       </c>
       <c r="D1263" s="4" t="inlineStr">
@@ -46884,7 +46884,7 @@
       </c>
       <c r="C1264" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-871</t>
         </is>
       </c>
       <c r="D1264" s="2" t="inlineStr">
@@ -46923,7 +46923,7 @@
       </c>
       <c r="C1265" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-875</t>
         </is>
       </c>
       <c r="D1265" s="4" t="inlineStr">
@@ -46962,7 +46962,7 @@
       </c>
       <c r="C1266" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-875</t>
         </is>
       </c>
       <c r="D1266" s="2" t="inlineStr">
@@ -47001,7 +47001,7 @@
       </c>
       <c r="C1267" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-876</t>
         </is>
       </c>
       <c r="D1267" s="4" t="inlineStr">
@@ -47040,7 +47040,7 @@
       </c>
       <c r="C1268" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-876</t>
         </is>
       </c>
       <c r="D1268" s="2" t="inlineStr">
@@ -47079,7 +47079,7 @@
       </c>
       <c r="C1269" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-880</t>
         </is>
       </c>
       <c r="D1269" s="4" t="inlineStr">
@@ -47118,7 +47118,7 @@
       </c>
       <c r="C1270" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-880</t>
         </is>
       </c>
       <c r="D1270" s="2" t="inlineStr">
@@ -47157,7 +47157,7 @@
       </c>
       <c r="C1271" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-881</t>
         </is>
       </c>
       <c r="D1271" s="4" t="inlineStr">
@@ -47196,7 +47196,7 @@
       </c>
       <c r="C1272" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-881</t>
         </is>
       </c>
       <c r="D1272" s="2" t="inlineStr">
@@ -47235,7 +47235,7 @@
       </c>
       <c r="C1273" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-885</t>
         </is>
       </c>
       <c r="D1273" s="4" t="inlineStr">
@@ -47274,7 +47274,7 @@
       </c>
       <c r="C1274" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-885</t>
         </is>
       </c>
       <c r="D1274" s="2" t="inlineStr">
@@ -47313,7 +47313,7 @@
       </c>
       <c r="C1275" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-886</t>
         </is>
       </c>
       <c r="D1275" s="4" t="inlineStr">
@@ -47352,7 +47352,7 @@
       </c>
       <c r="C1276" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>S-886</t>
         </is>
       </c>
       <c r="D1276" s="2" t="inlineStr">
@@ -47391,7 +47391,7 @@
       </c>
       <c r="C1277" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-405</t>
         </is>
       </c>
       <c r="D1277" s="4" t="inlineStr"/>
@@ -47426,7 +47426,7 @@
       </c>
       <c r="C1278" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-405</t>
         </is>
       </c>
       <c r="D1278" s="2" t="inlineStr"/>
@@ -47461,7 +47461,7 @@
       </c>
       <c r="C1279" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-405</t>
         </is>
       </c>
       <c r="D1279" s="4" t="inlineStr"/>
@@ -47496,7 +47496,7 @@
       </c>
       <c r="C1280" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-405</t>
         </is>
       </c>
       <c r="D1280" s="2" t="inlineStr"/>
@@ -47531,7 +47531,7 @@
       </c>
       <c r="C1281" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-405</t>
         </is>
       </c>
       <c r="D1281" s="4" t="inlineStr"/>
@@ -47566,7 +47566,7 @@
       </c>
       <c r="C1282" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-505</t>
         </is>
       </c>
       <c r="D1282" s="2" t="inlineStr"/>
@@ -47601,7 +47601,7 @@
       </c>
       <c r="C1283" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-505</t>
         </is>
       </c>
       <c r="D1283" s="4" t="inlineStr"/>
@@ -47636,7 +47636,7 @@
       </c>
       <c r="C1284" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-505</t>
         </is>
       </c>
       <c r="D1284" s="2" t="inlineStr"/>
@@ -47671,7 +47671,7 @@
       </c>
       <c r="C1285" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-505</t>
         </is>
       </c>
       <c r="D1285" s="4" t="inlineStr"/>
@@ -47706,7 +47706,7 @@
       </c>
       <c r="C1286" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-505</t>
         </is>
       </c>
       <c r="D1286" s="2" t="inlineStr"/>
@@ -47741,7 +47741,7 @@
       </c>
       <c r="C1287" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-407</t>
         </is>
       </c>
       <c r="D1287" s="4" t="inlineStr"/>
@@ -47776,7 +47776,7 @@
       </c>
       <c r="C1288" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-407</t>
         </is>
       </c>
       <c r="D1288" s="2" t="inlineStr"/>
@@ -47811,7 +47811,7 @@
       </c>
       <c r="C1289" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-407</t>
         </is>
       </c>
       <c r="D1289" s="4" t="inlineStr"/>
@@ -47846,7 +47846,7 @@
       </c>
       <c r="C1290" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-407</t>
         </is>
       </c>
       <c r="D1290" s="2" t="inlineStr"/>
@@ -47881,7 +47881,7 @@
       </c>
       <c r="C1291" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-407</t>
         </is>
       </c>
       <c r="D1291" s="4" t="inlineStr"/>
@@ -47916,7 +47916,7 @@
       </c>
       <c r="C1292" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-409</t>
         </is>
       </c>
       <c r="D1292" s="2" t="inlineStr"/>
@@ -47951,7 +47951,7 @@
       </c>
       <c r="C1293" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-409</t>
         </is>
       </c>
       <c r="D1293" s="4" t="inlineStr"/>
@@ -47986,7 +47986,7 @@
       </c>
       <c r="C1294" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-409</t>
         </is>
       </c>
       <c r="D1294" s="2" t="inlineStr"/>
@@ -48021,7 +48021,7 @@
       </c>
       <c r="C1295" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-409</t>
         </is>
       </c>
       <c r="D1295" s="4" t="inlineStr"/>
@@ -48056,7 +48056,7 @@
       </c>
       <c r="C1296" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-409</t>
         </is>
       </c>
       <c r="D1296" s="2" t="inlineStr"/>
@@ -48091,7 +48091,7 @@
       </c>
       <c r="C1297" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-410</t>
         </is>
       </c>
       <c r="D1297" s="4" t="inlineStr"/>
@@ -48126,7 +48126,7 @@
       </c>
       <c r="C1298" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-410</t>
         </is>
       </c>
       <c r="D1298" s="2" t="inlineStr"/>
@@ -48161,7 +48161,7 @@
       </c>
       <c r="C1299" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-410</t>
         </is>
       </c>
       <c r="D1299" s="4" t="inlineStr"/>
@@ -48196,7 +48196,7 @@
       </c>
       <c r="C1300" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-410</t>
         </is>
       </c>
       <c r="D1300" s="2" t="inlineStr"/>
@@ -48231,7 +48231,7 @@
       </c>
       <c r="C1301" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-410</t>
         </is>
       </c>
       <c r="D1301" s="4" t="inlineStr"/>
@@ -48266,7 +48266,7 @@
       </c>
       <c r="C1302" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-413</t>
         </is>
       </c>
       <c r="D1302" s="2" t="inlineStr"/>
@@ -48301,7 +48301,7 @@
       </c>
       <c r="C1303" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-413</t>
         </is>
       </c>
       <c r="D1303" s="4" t="inlineStr"/>
@@ -48336,7 +48336,7 @@
       </c>
       <c r="C1304" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-413</t>
         </is>
       </c>
       <c r="D1304" s="2" t="inlineStr"/>
@@ -48371,7 +48371,7 @@
       </c>
       <c r="C1305" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-413</t>
         </is>
       </c>
       <c r="D1305" s="4" t="inlineStr"/>
@@ -48406,7 +48406,7 @@
       </c>
       <c r="C1306" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-413</t>
         </is>
       </c>
       <c r="D1306" s="2" t="inlineStr"/>
@@ -48441,7 +48441,7 @@
       </c>
       <c r="C1307" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-507</t>
         </is>
       </c>
       <c r="D1307" s="4" t="inlineStr"/>
@@ -48476,7 +48476,7 @@
       </c>
       <c r="C1308" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-507</t>
         </is>
       </c>
       <c r="D1308" s="2" t="inlineStr"/>
@@ -48511,7 +48511,7 @@
       </c>
       <c r="C1309" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-507</t>
         </is>
       </c>
       <c r="D1309" s="4" t="inlineStr"/>
@@ -48546,7 +48546,7 @@
       </c>
       <c r="C1310" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-507</t>
         </is>
       </c>
       <c r="D1310" s="2" t="inlineStr"/>
@@ -48581,7 +48581,7 @@
       </c>
       <c r="C1311" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-507</t>
         </is>
       </c>
       <c r="D1311" s="4" t="inlineStr"/>
@@ -48616,7 +48616,7 @@
       </c>
       <c r="C1312" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-508</t>
         </is>
       </c>
       <c r="D1312" s="2" t="inlineStr"/>
@@ -48651,7 +48651,7 @@
       </c>
       <c r="C1313" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-508</t>
         </is>
       </c>
       <c r="D1313" s="4" t="inlineStr"/>
@@ -48686,7 +48686,7 @@
       </c>
       <c r="C1314" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-508</t>
         </is>
       </c>
       <c r="D1314" s="2" t="inlineStr"/>
@@ -48721,7 +48721,7 @@
       </c>
       <c r="C1315" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-508</t>
         </is>
       </c>
       <c r="D1315" s="4" t="inlineStr"/>
@@ -48756,7 +48756,7 @@
       </c>
       <c r="C1316" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-508</t>
         </is>
       </c>
       <c r="D1316" s="2" t="inlineStr"/>
@@ -48791,7 +48791,7 @@
       </c>
       <c r="C1317" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-513</t>
         </is>
       </c>
       <c r="D1317" s="4" t="inlineStr"/>
@@ -48826,7 +48826,7 @@
       </c>
       <c r="C1318" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-513</t>
         </is>
       </c>
       <c r="D1318" s="2" t="inlineStr"/>
@@ -48861,7 +48861,7 @@
       </c>
       <c r="C1319" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-513</t>
         </is>
       </c>
       <c r="D1319" s="4" t="inlineStr"/>
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C1320" s="2" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-513</t>
         </is>
       </c>
       <c r="D1320" s="2" t="inlineStr"/>
@@ -48931,7 +48931,7 @@
       </c>
       <c r="C1321" s="4" t="inlineStr">
         <is>
-          <t>WHPX</t>
+          <t>WHPX-513</t>
         </is>
       </c>
       <c r="D1321" s="4" t="inlineStr"/>
@@ -48966,7 +48966,7 @@
       </c>
       <c r="C1322" s="2" t="inlineStr">
         <is>
-          <t>SJ-E</t>
+          <t>SJ-E-all types</t>
         </is>
       </c>
       <c r="D1322" s="2" t="inlineStr"/>
@@ -49001,7 +49001,7 @@
       </c>
       <c r="C1323" s="4" t="inlineStr">
         <is>
-          <t>SJ-G</t>
+          <t>SJ-G-all types</t>
         </is>
       </c>
       <c r="D1323" s="4" t="inlineStr"/>
@@ -49071,7 +49071,7 @@
       </c>
       <c r="C1325" s="4" t="inlineStr">
         <is>
-          <t>OSA</t>
+          <t>OSA-7</t>
         </is>
       </c>
       <c r="D1325" s="4" t="inlineStr"/>
@@ -49106,7 +49106,7 @@
       </c>
       <c r="C1326" s="2" t="inlineStr">
         <is>
-          <t>OSA</t>
+          <t>OSA-7</t>
         </is>
       </c>
       <c r="D1326" s="2" t="inlineStr"/>
@@ -49141,7 +49141,7 @@
       </c>
       <c r="C1327" s="4" t="inlineStr">
         <is>
-          <t>OSA</t>
+          <t>OSA-20</t>
         </is>
       </c>
       <c r="D1327" s="4" t="inlineStr"/>
@@ -49176,7 +49176,7 @@
       </c>
       <c r="C1328" s="2" t="inlineStr">
         <is>
-          <t>OSA</t>
+          <t>OSA-35</t>
         </is>
       </c>
       <c r="D1328" s="2" t="inlineStr"/>
@@ -49211,7 +49211,7 @@
       </c>
       <c r="C1329" s="4" t="inlineStr">
         <is>
-          <t>OSB</t>
+          <t>OSB-20</t>
         </is>
       </c>
       <c r="D1329" s="4" t="inlineStr"/>
@@ -49246,7 +49246,7 @@
       </c>
       <c r="C1330" s="2" t="inlineStr">
         <is>
-          <t>OSB</t>
+          <t>OSB-30</t>
         </is>
       </c>
       <c r="D1330" s="2" t="inlineStr"/>
@@ -49281,7 +49281,7 @@
       </c>
       <c r="C1331" s="4" t="inlineStr">
         <is>
-          <t>OSB</t>
+          <t>OSB-35</t>
         </is>
       </c>
       <c r="D1331" s="4" t="inlineStr"/>
@@ -49316,7 +49316,7 @@
       </c>
       <c r="C1332" s="2" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-4</t>
         </is>
       </c>
       <c r="D1332" s="2" t="inlineStr"/>
@@ -49351,7 +49351,7 @@
       </c>
       <c r="C1333" s="4" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-4</t>
         </is>
       </c>
       <c r="D1333" s="4" t="inlineStr"/>
@@ -49386,7 +49386,7 @@
       </c>
       <c r="C1334" s="2" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-5</t>
         </is>
       </c>
       <c r="D1334" s="2" t="inlineStr"/>
@@ -49421,7 +49421,7 @@
       </c>
       <c r="C1335" s="4" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-5</t>
         </is>
       </c>
       <c r="D1335" s="4" t="inlineStr"/>
@@ -49456,7 +49456,7 @@
       </c>
       <c r="C1336" s="2" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-15</t>
         </is>
       </c>
       <c r="D1336" s="2" t="inlineStr"/>
@@ -49491,7 +49491,7 @@
       </c>
       <c r="C1337" s="4" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-18</t>
         </is>
       </c>
       <c r="D1337" s="4" t="inlineStr"/>
@@ -49526,7 +49526,7 @@
       </c>
       <c r="C1338" s="2" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-25</t>
         </is>
       </c>
       <c r="D1338" s="2" t="inlineStr"/>
@@ -49561,7 +49561,7 @@
       </c>
       <c r="C1339" s="4" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-30</t>
         </is>
       </c>
       <c r="D1339" s="4" t="inlineStr"/>
@@ -49596,7 +49596,7 @@
       </c>
       <c r="C1340" s="2" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-40</t>
         </is>
       </c>
       <c r="D1340" s="2" t="inlineStr"/>
@@ -49631,7 +49631,7 @@
       </c>
       <c r="C1341" s="4" t="inlineStr">
         <is>
-          <t>OSC</t>
+          <t>OSC-50</t>
         </is>
       </c>
       <c r="D1341" s="4" t="inlineStr"/>
@@ -49666,7 +49666,7 @@
       </c>
       <c r="C1342" s="2" t="inlineStr">
         <is>
-          <t>OSD</t>
+          <t>OSD-all types</t>
         </is>
       </c>
       <c r="D1342" s="2" t="inlineStr"/>
@@ -49701,7 +49701,7 @@
       </c>
       <c r="C1343" s="4" t="inlineStr">
         <is>
-          <t>OSD</t>
+          <t>OSD-all types</t>
         </is>
       </c>
       <c r="D1343" s="4" t="inlineStr"/>
@@ -49736,7 +49736,7 @@
       </c>
       <c r="C1344" s="2" t="inlineStr">
         <is>
-          <t>OSE</t>
+          <t>OSE-all types</t>
         </is>
       </c>
       <c r="D1344" s="2" t="inlineStr"/>
@@ -49771,7 +49771,7 @@
       </c>
       <c r="C1345" s="4" t="inlineStr">
         <is>
-          <t>OSE</t>
+          <t>OSE-all types</t>
         </is>
       </c>
       <c r="D1345" s="4" t="inlineStr"/>
@@ -49806,7 +49806,7 @@
       </c>
       <c r="C1346" s="2" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-2</t>
         </is>
       </c>
       <c r="D1346" s="2" t="inlineStr"/>
@@ -49841,7 +49841,7 @@
       </c>
       <c r="C1347" s="4" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-7</t>
         </is>
       </c>
       <c r="D1347" s="4" t="inlineStr"/>
@@ -49876,7 +49876,7 @@
       </c>
       <c r="C1348" s="2" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-14</t>
         </is>
       </c>
       <c r="D1348" s="2" t="inlineStr"/>
@@ -49911,7 +49911,7 @@
       </c>
       <c r="C1349" s="4" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-14</t>
         </is>
       </c>
       <c r="D1349" s="4" t="inlineStr"/>
@@ -49946,7 +49946,7 @@
       </c>
       <c r="C1350" s="2" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-14</t>
         </is>
       </c>
       <c r="D1350" s="2" t="inlineStr"/>
@@ -49981,7 +49981,7 @@
       </c>
       <c r="C1351" s="4" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-18</t>
         </is>
       </c>
       <c r="D1351" s="4" t="inlineStr"/>
@@ -50016,7 +50016,7 @@
       </c>
       <c r="C1352" s="2" t="inlineStr">
         <is>
-          <t>OTA</t>
+          <t>OTA-30</t>
         </is>
       </c>
       <c r="D1352" s="2" t="inlineStr"/>
@@ -50051,7 +50051,7 @@
       </c>
       <c r="C1353" s="4" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-1</t>
         </is>
       </c>
       <c r="D1353" s="4" t="inlineStr"/>
@@ -50086,7 +50086,7 @@
       </c>
       <c r="C1354" s="2" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-1</t>
         </is>
       </c>
       <c r="D1354" s="2" t="inlineStr"/>
@@ -50121,7 +50121,7 @@
       </c>
       <c r="C1355" s="4" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-3</t>
         </is>
       </c>
       <c r="D1355" s="4" t="inlineStr"/>
@@ -50156,7 +50156,7 @@
       </c>
       <c r="C1356" s="2" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-3</t>
         </is>
       </c>
       <c r="D1356" s="2" t="inlineStr"/>
@@ -50191,7 +50191,7 @@
       </c>
       <c r="C1357" s="4" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-9</t>
         </is>
       </c>
       <c r="D1357" s="4" t="inlineStr"/>
@@ -50226,7 +50226,7 @@
       </c>
       <c r="C1358" s="2" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-9</t>
         </is>
       </c>
       <c r="D1358" s="2" t="inlineStr"/>
@@ -50261,7 +50261,7 @@
       </c>
       <c r="C1359" s="4" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-18</t>
         </is>
       </c>
       <c r="D1359" s="4" t="inlineStr"/>
@@ -50296,7 +50296,7 @@
       </c>
       <c r="C1360" s="2" t="inlineStr">
         <is>
-          <t>OTB</t>
+          <t>OTB-35</t>
         </is>
       </c>
       <c r="D1360" s="2" t="inlineStr"/>
@@ -50331,7 +50331,7 @@
       </c>
       <c r="C1361" s="4" t="inlineStr">
         <is>
-          <t>OTC</t>
+          <t>OTC-all types</t>
         </is>
       </c>
       <c r="D1361" s="4" t="inlineStr"/>
@@ -50366,7 +50366,7 @@
       </c>
       <c r="C1362" s="2" t="inlineStr">
         <is>
-          <t>OTC</t>
+          <t>OTC-all types</t>
         </is>
       </c>
       <c r="D1362" s="2" t="inlineStr"/>
@@ -51444,7 +51444,7 @@
       </c>
       <c r="C1392" s="2" t="inlineStr">
         <is>
-          <t>VTR..0  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..0 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1392" s="2" t="inlineStr">
@@ -51483,7 +51483,7 @@
       </c>
       <c r="C1393" s="4" t="inlineStr">
         <is>
-          <t>VTR..0  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..0 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1393" s="4" t="inlineStr">
@@ -51522,7 +51522,7 @@
       </c>
       <c r="C1394" s="2" t="inlineStr">
         <is>
-          <t>VTR..0  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..0 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1394" s="2" t="inlineStr">
@@ -51561,7 +51561,7 @@
       </c>
       <c r="C1395" s="4" t="inlineStr">
         <is>
-          <t>VTR..1  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..1 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1395" s="4" t="inlineStr">
@@ -51600,7 +51600,7 @@
       </c>
       <c r="C1396" s="2" t="inlineStr">
         <is>
-          <t>VTR..1  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..1 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1396" s="2" t="inlineStr">
@@ -51639,7 +51639,7 @@
       </c>
       <c r="C1397" s="4" t="inlineStr">
         <is>
-          <t>VTR..1  With rolling contact bearings and INTEGRAL lubrication</t>
+          <t>VTR..1 With rolling contact bearings and INTEGRAL lubrication</t>
         </is>
       </c>
       <c r="D1397" s="4" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-30 12:02
</commit_message>
<xml_diff>
--- a/output/oem_master.xlsx
+++ b/output/oem_master.xlsx
@@ -36086,7 +36086,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>BWPX-307</t>
+          <t>BWPX 307</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr"/>
@@ -36121,7 +36121,7 @@
       </c>
       <c r="C963" s="4" t="inlineStr">
         <is>
-          <t>BWPX-307</t>
+          <t>BWPX 307</t>
         </is>
       </c>
       <c r="D963" s="4" t="inlineStr"/>
@@ -36156,7 +36156,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>BWPX-307</t>
+          <t>BWPX 307</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr"/>
@@ -36191,7 +36191,7 @@
       </c>
       <c r="C965" s="4" t="inlineStr">
         <is>
-          <t>BWPX-307</t>
+          <t>BWPX 307</t>
         </is>
       </c>
       <c r="D965" s="4" t="inlineStr"/>
@@ -36226,7 +36226,7 @@
       </c>
       <c r="C966" s="2" t="inlineStr">
         <is>
-          <t>FOPX-605</t>
+          <t>FOPX 605</t>
         </is>
       </c>
       <c r="D966" s="2" t="inlineStr"/>
@@ -36261,7 +36261,7 @@
       </c>
       <c r="C967" s="4" t="inlineStr">
         <is>
-          <t>FOPX-605</t>
+          <t>FOPX 605</t>
         </is>
       </c>
       <c r="D967" s="4" t="inlineStr"/>
@@ -36296,7 +36296,7 @@
       </c>
       <c r="C968" s="2" t="inlineStr">
         <is>
-          <t>FOPX-605</t>
+          <t>FOPX 605</t>
         </is>
       </c>
       <c r="D968" s="2" t="inlineStr"/>
@@ -36331,7 +36331,7 @@
       </c>
       <c r="C969" s="4" t="inlineStr">
         <is>
-          <t>FOPX-605</t>
+          <t>FOPX 605</t>
         </is>
       </c>
       <c r="D969" s="4" t="inlineStr"/>
@@ -36366,7 +36366,7 @@
       </c>
       <c r="C970" s="2" t="inlineStr">
         <is>
-          <t>FOPX-605</t>
+          <t>FOPX 605</t>
         </is>
       </c>
       <c r="D970" s="2" t="inlineStr"/>
@@ -36401,7 +36401,7 @@
       </c>
       <c r="C971" s="4" t="inlineStr">
         <is>
-          <t>FOPX-607</t>
+          <t>FOPX 607</t>
         </is>
       </c>
       <c r="D971" s="4" t="inlineStr"/>
@@ -36436,7 +36436,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>FOPX-607</t>
+          <t>FOPX 607</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr"/>
@@ -36471,7 +36471,7 @@
       </c>
       <c r="C973" s="4" t="inlineStr">
         <is>
-          <t>FOPX-607</t>
+          <t>FOPX 607</t>
         </is>
       </c>
       <c r="D973" s="4" t="inlineStr"/>
@@ -36506,7 +36506,7 @@
       </c>
       <c r="C974" s="2" t="inlineStr">
         <is>
-          <t>FOPX-607</t>
+          <t>FOPX 607</t>
         </is>
       </c>
       <c r="D974" s="2" t="inlineStr"/>
@@ -36541,7 +36541,7 @@
       </c>
       <c r="C975" s="4" t="inlineStr">
         <is>
-          <t>FOPX-607</t>
+          <t>FOPX 607</t>
         </is>
       </c>
       <c r="D975" s="4" t="inlineStr"/>
@@ -36576,7 +36576,7 @@
       </c>
       <c r="C976" s="2" t="inlineStr">
         <is>
-          <t>FOPX-609</t>
+          <t>FOPX 609</t>
         </is>
       </c>
       <c r="D976" s="2" t="inlineStr"/>
@@ -36611,7 +36611,7 @@
       </c>
       <c r="C977" s="4" t="inlineStr">
         <is>
-          <t>FOPX-609</t>
+          <t>FOPX 609</t>
         </is>
       </c>
       <c r="D977" s="4" t="inlineStr"/>
@@ -36646,7 +36646,7 @@
       </c>
       <c r="C978" s="2" t="inlineStr">
         <is>
-          <t>FOPX-609</t>
+          <t>FOPX 609</t>
         </is>
       </c>
       <c r="D978" s="2" t="inlineStr"/>
@@ -36681,7 +36681,7 @@
       </c>
       <c r="C979" s="4" t="inlineStr">
         <is>
-          <t>FOPX-609</t>
+          <t>FOPX 609</t>
         </is>
       </c>
       <c r="D979" s="4" t="inlineStr"/>
@@ -36716,7 +36716,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>FOPX-609</t>
+          <t>FOPX 609</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr"/>
@@ -36751,7 +36751,7 @@
       </c>
       <c r="C981" s="4" t="inlineStr">
         <is>
-          <t>FOPX-610</t>
+          <t>FOPX 610</t>
         </is>
       </c>
       <c r="D981" s="4" t="inlineStr"/>
@@ -36786,7 +36786,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>FOPX-610</t>
+          <t>FOPX 610</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr"/>
@@ -36821,7 +36821,7 @@
       </c>
       <c r="C983" s="4" t="inlineStr">
         <is>
-          <t>FOPX-610</t>
+          <t>FOPX 610</t>
         </is>
       </c>
       <c r="D983" s="4" t="inlineStr"/>
@@ -36856,7 +36856,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>FOPX-610</t>
+          <t>FOPX 610</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr"/>
@@ -36891,7 +36891,7 @@
       </c>
       <c r="C985" s="4" t="inlineStr">
         <is>
-          <t>FOPX-610</t>
+          <t>FOPX 610</t>
         </is>
       </c>
       <c r="D985" s="4" t="inlineStr"/>
@@ -36926,7 +36926,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>FOPX-611</t>
+          <t>FOPX 611</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr"/>
@@ -36961,7 +36961,7 @@
       </c>
       <c r="C987" s="4" t="inlineStr">
         <is>
-          <t>FOPX-611</t>
+          <t>FOPX 611</t>
         </is>
       </c>
       <c r="D987" s="4" t="inlineStr"/>
@@ -36996,7 +36996,7 @@
       </c>
       <c r="C988" s="2" t="inlineStr">
         <is>
-          <t>FOPX-611</t>
+          <t>FOPX 611</t>
         </is>
       </c>
       <c r="D988" s="2" t="inlineStr"/>
@@ -37031,7 +37031,7 @@
       </c>
       <c r="C989" s="4" t="inlineStr">
         <is>
-          <t>FOPX-611</t>
+          <t>FOPX 611</t>
         </is>
       </c>
       <c r="D989" s="4" t="inlineStr"/>
@@ -37066,7 +37066,7 @@
       </c>
       <c r="C990" s="2" t="inlineStr">
         <is>
-          <t>FOPX-611</t>
+          <t>FOPX 611</t>
         </is>
       </c>
       <c r="D990" s="2" t="inlineStr"/>
@@ -37101,7 +37101,7 @@
       </c>
       <c r="C991" s="4" t="inlineStr">
         <is>
-          <t>FOPX-613</t>
+          <t>FOPX 613</t>
         </is>
       </c>
       <c r="D991" s="4" t="inlineStr"/>
@@ -37136,7 +37136,7 @@
       </c>
       <c r="C992" s="2" t="inlineStr">
         <is>
-          <t>FOPX-613</t>
+          <t>FOPX 613</t>
         </is>
       </c>
       <c r="D992" s="2" t="inlineStr"/>
@@ -37171,7 +37171,7 @@
       </c>
       <c r="C993" s="4" t="inlineStr">
         <is>
-          <t>FOPX-613</t>
+          <t>FOPX 613</t>
         </is>
       </c>
       <c r="D993" s="4" t="inlineStr"/>
@@ -37206,7 +37206,7 @@
       </c>
       <c r="C994" s="2" t="inlineStr">
         <is>
-          <t>FOPX-613</t>
+          <t>FOPX 613</t>
         </is>
       </c>
       <c r="D994" s="2" t="inlineStr"/>
@@ -37241,7 +37241,7 @@
       </c>
       <c r="C995" s="4" t="inlineStr">
         <is>
-          <t>FOPX-613</t>
+          <t>FOPX 613</t>
         </is>
       </c>
       <c r="D995" s="4" t="inlineStr"/>
@@ -37276,7 +37276,7 @@
       </c>
       <c r="C996" s="2" t="inlineStr">
         <is>
-          <t>FOPX-614</t>
+          <t>FOPX 614</t>
         </is>
       </c>
       <c r="D996" s="2" t="inlineStr"/>
@@ -37311,7 +37311,7 @@
       </c>
       <c r="C997" s="4" t="inlineStr">
         <is>
-          <t>FOPX-614</t>
+          <t>FOPX 614</t>
         </is>
       </c>
       <c r="D997" s="4" t="inlineStr"/>
@@ -37346,7 +37346,7 @@
       </c>
       <c r="C998" s="2" t="inlineStr">
         <is>
-          <t>FOPX-614</t>
+          <t>FOPX 614</t>
         </is>
       </c>
       <c r="D998" s="2" t="inlineStr"/>
@@ -37381,7 +37381,7 @@
       </c>
       <c r="C999" s="4" t="inlineStr">
         <is>
-          <t>FOPX-614</t>
+          <t>FOPX 614</t>
         </is>
       </c>
       <c r="D999" s="4" t="inlineStr"/>
@@ -37416,7 +37416,7 @@
       </c>
       <c r="C1000" s="2" t="inlineStr">
         <is>
-          <t>FOPX-614</t>
+          <t>FOPX 614</t>
         </is>
       </c>
       <c r="D1000" s="2" t="inlineStr"/>
@@ -37451,7 +37451,7 @@
       </c>
       <c r="C1001" s="4" t="inlineStr">
         <is>
-          <t>LOPX-705</t>
+          <t>LOPX 705</t>
         </is>
       </c>
       <c r="D1001" s="4" t="inlineStr"/>
@@ -37486,7 +37486,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>LOPX-705</t>
+          <t>LOPX 705</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr"/>
@@ -37521,7 +37521,7 @@
       </c>
       <c r="C1003" s="4" t="inlineStr">
         <is>
-          <t>LOPX-705</t>
+          <t>LOPX 705</t>
         </is>
       </c>
       <c r="D1003" s="4" t="inlineStr"/>
@@ -37556,7 +37556,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>LOPX-705</t>
+          <t>LOPX 705</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr"/>
@@ -37591,7 +37591,7 @@
       </c>
       <c r="C1005" s="4" t="inlineStr">
         <is>
-          <t>LOPX-705</t>
+          <t>LOPX 705</t>
         </is>
       </c>
       <c r="D1005" s="4" t="inlineStr"/>
@@ -37626,7 +37626,7 @@
       </c>
       <c r="C1006" s="2" t="inlineStr">
         <is>
-          <t>LOPX-707</t>
+          <t>LOPX 707</t>
         </is>
       </c>
       <c r="D1006" s="2" t="inlineStr"/>
@@ -37661,7 +37661,7 @@
       </c>
       <c r="C1007" s="4" t="inlineStr">
         <is>
-          <t>LOPX-707</t>
+          <t>LOPX 707</t>
         </is>
       </c>
       <c r="D1007" s="4" t="inlineStr"/>
@@ -37696,7 +37696,7 @@
       </c>
       <c r="C1008" s="2" t="inlineStr">
         <is>
-          <t>LOPX-707</t>
+          <t>LOPX 707</t>
         </is>
       </c>
       <c r="D1008" s="2" t="inlineStr"/>
@@ -37731,7 +37731,7 @@
       </c>
       <c r="C1009" s="4" t="inlineStr">
         <is>
-          <t>LOPX-707</t>
+          <t>LOPX 707</t>
         </is>
       </c>
       <c r="D1009" s="4" t="inlineStr"/>
@@ -37766,7 +37766,7 @@
       </c>
       <c r="C1010" s="2" t="inlineStr">
         <is>
-          <t>LOPX-707</t>
+          <t>LOPX 707</t>
         </is>
       </c>
       <c r="D1010" s="2" t="inlineStr"/>
@@ -37801,7 +37801,7 @@
       </c>
       <c r="C1011" s="4" t="inlineStr">
         <is>
-          <t>LOPX-709</t>
+          <t>LOPX 709</t>
         </is>
       </c>
       <c r="D1011" s="4" t="inlineStr"/>
@@ -37836,7 +37836,7 @@
       </c>
       <c r="C1012" s="2" t="inlineStr">
         <is>
-          <t>LOPX-709</t>
+          <t>LOPX 709</t>
         </is>
       </c>
       <c r="D1012" s="2" t="inlineStr"/>
@@ -37871,7 +37871,7 @@
       </c>
       <c r="C1013" s="4" t="inlineStr">
         <is>
-          <t>LOPX-709</t>
+          <t>LOPX 709</t>
         </is>
       </c>
       <c r="D1013" s="4" t="inlineStr"/>
@@ -37906,7 +37906,7 @@
       </c>
       <c r="C1014" s="2" t="inlineStr">
         <is>
-          <t>LOPX-709</t>
+          <t>LOPX 709</t>
         </is>
       </c>
       <c r="D1014" s="2" t="inlineStr"/>
@@ -37941,7 +37941,7 @@
       </c>
       <c r="C1015" s="4" t="inlineStr">
         <is>
-          <t>LOPX-709</t>
+          <t>LOPX 709</t>
         </is>
       </c>
       <c r="D1015" s="4" t="inlineStr"/>
@@ -37976,7 +37976,7 @@
       </c>
       <c r="C1016" s="2" t="inlineStr">
         <is>
-          <t>LOPX-710</t>
+          <t>LOPX 710</t>
         </is>
       </c>
       <c r="D1016" s="2" t="inlineStr"/>
@@ -38011,7 +38011,7 @@
       </c>
       <c r="C1017" s="4" t="inlineStr">
         <is>
-          <t>LOPX-710</t>
+          <t>LOPX 710</t>
         </is>
       </c>
       <c r="D1017" s="4" t="inlineStr"/>
@@ -38046,7 +38046,7 @@
       </c>
       <c r="C1018" s="2" t="inlineStr">
         <is>
-          <t>LOPX-710</t>
+          <t>LOPX 710</t>
         </is>
       </c>
       <c r="D1018" s="2" t="inlineStr"/>
@@ -38081,7 +38081,7 @@
       </c>
       <c r="C1019" s="4" t="inlineStr">
         <is>
-          <t>LOPX-710</t>
+          <t>LOPX 710</t>
         </is>
       </c>
       <c r="D1019" s="4" t="inlineStr"/>
@@ -38116,7 +38116,7 @@
       </c>
       <c r="C1020" s="2" t="inlineStr">
         <is>
-          <t>LOPX-710</t>
+          <t>LOPX 710</t>
         </is>
       </c>
       <c r="D1020" s="2" t="inlineStr"/>
@@ -38151,7 +38151,7 @@
       </c>
       <c r="C1021" s="4" t="inlineStr">
         <is>
-          <t>LOPX-711</t>
+          <t>LOPX 711</t>
         </is>
       </c>
       <c r="D1021" s="4" t="inlineStr"/>
@@ -38186,7 +38186,7 @@
       </c>
       <c r="C1022" s="2" t="inlineStr">
         <is>
-          <t>LOPX-711</t>
+          <t>LOPX 711</t>
         </is>
       </c>
       <c r="D1022" s="2" t="inlineStr"/>
@@ -38221,7 +38221,7 @@
       </c>
       <c r="C1023" s="4" t="inlineStr">
         <is>
-          <t>LOPX-711</t>
+          <t>LOPX 711</t>
         </is>
       </c>
       <c r="D1023" s="4" t="inlineStr"/>
@@ -38256,7 +38256,7 @@
       </c>
       <c r="C1024" s="2" t="inlineStr">
         <is>
-          <t>LOPX-711</t>
+          <t>LOPX 711</t>
         </is>
       </c>
       <c r="D1024" s="2" t="inlineStr"/>
@@ -38291,7 +38291,7 @@
       </c>
       <c r="C1025" s="4" t="inlineStr">
         <is>
-          <t>LOPX-711</t>
+          <t>LOPX 711</t>
         </is>
       </c>
       <c r="D1025" s="4" t="inlineStr"/>
@@ -38326,7 +38326,7 @@
       </c>
       <c r="C1026" s="2" t="inlineStr">
         <is>
-          <t>LOPX-713</t>
+          <t>LOPX 713</t>
         </is>
       </c>
       <c r="D1026" s="2" t="inlineStr"/>
@@ -38361,7 +38361,7 @@
       </c>
       <c r="C1027" s="4" t="inlineStr">
         <is>
-          <t>LOPX-713</t>
+          <t>LOPX 713</t>
         </is>
       </c>
       <c r="D1027" s="4" t="inlineStr"/>
@@ -38396,7 +38396,7 @@
       </c>
       <c r="C1028" s="2" t="inlineStr">
         <is>
-          <t>LOPX-713</t>
+          <t>LOPX 713</t>
         </is>
       </c>
       <c r="D1028" s="2" t="inlineStr"/>
@@ -38431,7 +38431,7 @@
       </c>
       <c r="C1029" s="4" t="inlineStr">
         <is>
-          <t>LOPX-713</t>
+          <t>LOPX 713</t>
         </is>
       </c>
       <c r="D1029" s="4" t="inlineStr"/>
@@ -38466,7 +38466,7 @@
       </c>
       <c r="C1030" s="2" t="inlineStr">
         <is>
-          <t>LOPX-713</t>
+          <t>LOPX 713</t>
         </is>
       </c>
       <c r="D1030" s="2" t="inlineStr"/>
@@ -38501,7 +38501,7 @@
       </c>
       <c r="C1031" s="4" t="inlineStr">
         <is>
-          <t>LOPX-714</t>
+          <t>LOPX 714</t>
         </is>
       </c>
       <c r="D1031" s="4" t="inlineStr"/>
@@ -38536,7 +38536,7 @@
       </c>
       <c r="C1032" s="2" t="inlineStr">
         <is>
-          <t>LOPX-714</t>
+          <t>LOPX 714</t>
         </is>
       </c>
       <c r="D1032" s="2" t="inlineStr"/>
@@ -38571,7 +38571,7 @@
       </c>
       <c r="C1033" s="4" t="inlineStr">
         <is>
-          <t>LOPX-714</t>
+          <t>LOPX 714</t>
         </is>
       </c>
       <c r="D1033" s="4" t="inlineStr"/>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="C1034" s="2" t="inlineStr">
         <is>
-          <t>LOPX-714</t>
+          <t>LOPX 714</t>
         </is>
       </c>
       <c r="D1034" s="2" t="inlineStr"/>
@@ -38641,7 +38641,7 @@
       </c>
       <c r="C1035" s="4" t="inlineStr">
         <is>
-          <t>LOPX-714</t>
+          <t>LOPX 714</t>
         </is>
       </c>
       <c r="D1035" s="4" t="inlineStr"/>
@@ -38676,7 +38676,7 @@
       </c>
       <c r="C1036" s="2" t="inlineStr">
         <is>
-          <t>MAB-102</t>
+          <t>MAB 102</t>
         </is>
       </c>
       <c r="D1036" s="2" t="inlineStr"/>
@@ -38711,7 +38711,7 @@
       </c>
       <c r="C1037" s="4" t="inlineStr">
         <is>
-          <t>MAB-102</t>
+          <t>MAB 102</t>
         </is>
       </c>
       <c r="D1037" s="4" t="inlineStr"/>
@@ -38746,7 +38746,7 @@
       </c>
       <c r="C1038" s="2" t="inlineStr">
         <is>
-          <t>MAB-102</t>
+          <t>MAB 102</t>
         </is>
       </c>
       <c r="D1038" s="2" t="inlineStr"/>
@@ -38781,7 +38781,7 @@
       </c>
       <c r="C1039" s="4" t="inlineStr">
         <is>
-          <t>MAB-102</t>
+          <t>MAB 102</t>
         </is>
       </c>
       <c r="D1039" s="4" t="inlineStr"/>
@@ -38816,7 +38816,7 @@
       </c>
       <c r="C1040" s="2" t="inlineStr">
         <is>
-          <t>MAB-102</t>
+          <t>MAB 102</t>
         </is>
       </c>
       <c r="D1040" s="2" t="inlineStr"/>
@@ -38851,7 +38851,7 @@
       </c>
       <c r="C1041" s="4" t="inlineStr">
         <is>
-          <t>MAB-103</t>
+          <t>MAB 103</t>
         </is>
       </c>
       <c r="D1041" s="4" t="inlineStr"/>
@@ -38886,7 +38886,7 @@
       </c>
       <c r="C1042" s="2" t="inlineStr">
         <is>
-          <t>MAB-103</t>
+          <t>MAB 103</t>
         </is>
       </c>
       <c r="D1042" s="2" t="inlineStr"/>
@@ -38921,7 +38921,7 @@
       </c>
       <c r="C1043" s="4" t="inlineStr">
         <is>
-          <t>MAB-103</t>
+          <t>MAB 103</t>
         </is>
       </c>
       <c r="D1043" s="4" t="inlineStr"/>
@@ -38956,7 +38956,7 @@
       </c>
       <c r="C1044" s="2" t="inlineStr">
         <is>
-          <t>MAB-103</t>
+          <t>MAB 103</t>
         </is>
       </c>
       <c r="D1044" s="2" t="inlineStr"/>
@@ -38991,7 +38991,7 @@
       </c>
       <c r="C1045" s="4" t="inlineStr">
         <is>
-          <t>MAB-103</t>
+          <t>MAB 103</t>
         </is>
       </c>
       <c r="D1045" s="4" t="inlineStr"/>
@@ -39026,7 +39026,7 @@
       </c>
       <c r="C1046" s="2" t="inlineStr">
         <is>
-          <t>MAB-104</t>
+          <t>MAB 104</t>
         </is>
       </c>
       <c r="D1046" s="2" t="inlineStr"/>
@@ -39061,7 +39061,7 @@
       </c>
       <c r="C1047" s="4" t="inlineStr">
         <is>
-          <t>MAB-104</t>
+          <t>MAB 104</t>
         </is>
       </c>
       <c r="D1047" s="4" t="inlineStr"/>
@@ -39096,7 +39096,7 @@
       </c>
       <c r="C1048" s="2" t="inlineStr">
         <is>
-          <t>MAB-104</t>
+          <t>MAB 104</t>
         </is>
       </c>
       <c r="D1048" s="2" t="inlineStr"/>
@@ -39131,7 +39131,7 @@
       </c>
       <c r="C1049" s="4" t="inlineStr">
         <is>
-          <t>MAB-104</t>
+          <t>MAB 104</t>
         </is>
       </c>
       <c r="D1049" s="4" t="inlineStr"/>
@@ -39166,7 +39166,7 @@
       </c>
       <c r="C1050" s="2" t="inlineStr">
         <is>
-          <t>MAB-104</t>
+          <t>MAB 104</t>
         </is>
       </c>
       <c r="D1050" s="2" t="inlineStr"/>
@@ -39201,7 +39201,7 @@
       </c>
       <c r="C1051" s="4" t="inlineStr">
         <is>
-          <t>MAB-204</t>
+          <t>MAB 204</t>
         </is>
       </c>
       <c r="D1051" s="4" t="inlineStr"/>
@@ -39236,7 +39236,7 @@
       </c>
       <c r="C1052" s="2" t="inlineStr">
         <is>
-          <t>MAB-204</t>
+          <t>MAB 204</t>
         </is>
       </c>
       <c r="D1052" s="2" t="inlineStr"/>
@@ -39271,7 +39271,7 @@
       </c>
       <c r="C1053" s="4" t="inlineStr">
         <is>
-          <t>MAB-204</t>
+          <t>MAB 204</t>
         </is>
       </c>
       <c r="D1053" s="4" t="inlineStr"/>
@@ -39306,7 +39306,7 @@
       </c>
       <c r="C1054" s="2" t="inlineStr">
         <is>
-          <t>MAB-204</t>
+          <t>MAB 204</t>
         </is>
       </c>
       <c r="D1054" s="2" t="inlineStr"/>
@@ -39341,7 +39341,7 @@
       </c>
       <c r="C1055" s="4" t="inlineStr">
         <is>
-          <t>MAB-204</t>
+          <t>MAB 204</t>
         </is>
       </c>
       <c r="D1055" s="4" t="inlineStr"/>
@@ -39376,7 +39376,7 @@
       </c>
       <c r="C1056" s="2" t="inlineStr">
         <is>
-          <t>MAB-205</t>
+          <t>MAB 205</t>
         </is>
       </c>
       <c r="D1056" s="2" t="inlineStr"/>
@@ -39411,7 +39411,7 @@
       </c>
       <c r="C1057" s="4" t="inlineStr">
         <is>
-          <t>MAB-205</t>
+          <t>MAB 205</t>
         </is>
       </c>
       <c r="D1057" s="4" t="inlineStr"/>
@@ -39446,7 +39446,7 @@
       </c>
       <c r="C1058" s="2" t="inlineStr">
         <is>
-          <t>MAB-205</t>
+          <t>MAB 205</t>
         </is>
       </c>
       <c r="D1058" s="2" t="inlineStr"/>
@@ -39481,7 +39481,7 @@
       </c>
       <c r="C1059" s="4" t="inlineStr">
         <is>
-          <t>MAB-205</t>
+          <t>MAB 205</t>
         </is>
       </c>
       <c r="D1059" s="4" t="inlineStr"/>
@@ -39516,7 +39516,7 @@
       </c>
       <c r="C1060" s="2" t="inlineStr">
         <is>
-          <t>MAB-205</t>
+          <t>MAB 205</t>
         </is>
       </c>
       <c r="D1060" s="2" t="inlineStr"/>
@@ -39551,7 +39551,7 @@
       </c>
       <c r="C1061" s="4" t="inlineStr">
         <is>
-          <t>MAB-206</t>
+          <t>MAB 206</t>
         </is>
       </c>
       <c r="D1061" s="4" t="inlineStr"/>
@@ -39586,7 +39586,7 @@
       </c>
       <c r="C1062" s="2" t="inlineStr">
         <is>
-          <t>MAB-206</t>
+          <t>MAB 206</t>
         </is>
       </c>
       <c r="D1062" s="2" t="inlineStr"/>
@@ -39621,7 +39621,7 @@
       </c>
       <c r="C1063" s="4" t="inlineStr">
         <is>
-          <t>MAB-206</t>
+          <t>MAB 206</t>
         </is>
       </c>
       <c r="D1063" s="4" t="inlineStr"/>
@@ -39656,7 +39656,7 @@
       </c>
       <c r="C1064" s="2" t="inlineStr">
         <is>
-          <t>MAB-206</t>
+          <t>MAB 206</t>
         </is>
       </c>
       <c r="D1064" s="2" t="inlineStr"/>
@@ -39691,7 +39691,7 @@
       </c>
       <c r="C1065" s="4" t="inlineStr">
         <is>
-          <t>MAB-206</t>
+          <t>MAB 206</t>
         </is>
       </c>
       <c r="D1065" s="4" t="inlineStr"/>
@@ -39726,7 +39726,7 @@
       </c>
       <c r="C1066" s="2" t="inlineStr">
         <is>
-          <t>MAB-207</t>
+          <t>MAB 207</t>
         </is>
       </c>
       <c r="D1066" s="2" t="inlineStr"/>
@@ -39761,7 +39761,7 @@
       </c>
       <c r="C1067" s="4" t="inlineStr">
         <is>
-          <t>MAB-207</t>
+          <t>MAB 207</t>
         </is>
       </c>
       <c r="D1067" s="4" t="inlineStr"/>
@@ -39796,7 +39796,7 @@
       </c>
       <c r="C1068" s="2" t="inlineStr">
         <is>
-          <t>MAB-207</t>
+          <t>MAB 207</t>
         </is>
       </c>
       <c r="D1068" s="2" t="inlineStr"/>
@@ -39831,7 +39831,7 @@
       </c>
       <c r="C1069" s="4" t="inlineStr">
         <is>
-          <t>MAB-207</t>
+          <t>MAB 207</t>
         </is>
       </c>
       <c r="D1069" s="4" t="inlineStr"/>
@@ -39866,7 +39866,7 @@
       </c>
       <c r="C1070" s="2" t="inlineStr">
         <is>
-          <t>MAB-207</t>
+          <t>MAB 207</t>
         </is>
       </c>
       <c r="D1070" s="2" t="inlineStr"/>
@@ -39901,7 +39901,7 @@
       </c>
       <c r="C1071" s="4" t="inlineStr">
         <is>
-          <t>MAB-209</t>
+          <t>MAB 209</t>
         </is>
       </c>
       <c r="D1071" s="4" t="inlineStr"/>
@@ -39936,7 +39936,7 @@
       </c>
       <c r="C1072" s="2" t="inlineStr">
         <is>
-          <t>MAB-209</t>
+          <t>MAB 209</t>
         </is>
       </c>
       <c r="D1072" s="2" t="inlineStr"/>
@@ -39971,7 +39971,7 @@
       </c>
       <c r="C1073" s="4" t="inlineStr">
         <is>
-          <t>MAB-209</t>
+          <t>MAB 209</t>
         </is>
       </c>
       <c r="D1073" s="4" t="inlineStr"/>
@@ -40006,7 +40006,7 @@
       </c>
       <c r="C1074" s="2" t="inlineStr">
         <is>
-          <t>MAB-209</t>
+          <t>MAB 209</t>
         </is>
       </c>
       <c r="D1074" s="2" t="inlineStr"/>
@@ -40041,7 +40041,7 @@
       </c>
       <c r="C1075" s="4" t="inlineStr">
         <is>
-          <t>MAB-209</t>
+          <t>MAB 209</t>
         </is>
       </c>
       <c r="D1075" s="4" t="inlineStr"/>
@@ -40076,7 +40076,7 @@
       </c>
       <c r="C1076" s="2" t="inlineStr">
         <is>
-          <t>MAPX-204</t>
+          <t>MAPX 204</t>
         </is>
       </c>
       <c r="D1076" s="2" t="inlineStr"/>
@@ -40111,7 +40111,7 @@
       </c>
       <c r="C1077" s="4" t="inlineStr">
         <is>
-          <t>MAPX-204</t>
+          <t>MAPX 204</t>
         </is>
       </c>
       <c r="D1077" s="4" t="inlineStr"/>
@@ -40146,7 +40146,7 @@
       </c>
       <c r="C1078" s="2" t="inlineStr">
         <is>
-          <t>MAPX-204</t>
+          <t>MAPX 204</t>
         </is>
       </c>
       <c r="D1078" s="2" t="inlineStr"/>
@@ -40181,7 +40181,7 @@
       </c>
       <c r="C1079" s="4" t="inlineStr">
         <is>
-          <t>MAPX-204</t>
+          <t>MAPX 204</t>
         </is>
       </c>
       <c r="D1079" s="4" t="inlineStr"/>
@@ -40216,7 +40216,7 @@
       </c>
       <c r="C1080" s="2" t="inlineStr">
         <is>
-          <t>MAPX-204</t>
+          <t>MAPX 204</t>
         </is>
       </c>
       <c r="D1080" s="2" t="inlineStr"/>
@@ -40251,7 +40251,7 @@
       </c>
       <c r="C1081" s="4" t="inlineStr">
         <is>
-          <t>MAPX-205</t>
+          <t>MAPX 205</t>
         </is>
       </c>
       <c r="D1081" s="4" t="inlineStr"/>
@@ -40286,7 +40286,7 @@
       </c>
       <c r="C1082" s="2" t="inlineStr">
         <is>
-          <t>MAPX-205</t>
+          <t>MAPX 205</t>
         </is>
       </c>
       <c r="D1082" s="2" t="inlineStr"/>
@@ -40321,7 +40321,7 @@
       </c>
       <c r="C1083" s="4" t="inlineStr">
         <is>
-          <t>MAPX-205</t>
+          <t>MAPX 205</t>
         </is>
       </c>
       <c r="D1083" s="4" t="inlineStr"/>
@@ -40356,7 +40356,7 @@
       </c>
       <c r="C1084" s="2" t="inlineStr">
         <is>
-          <t>MAPX-205</t>
+          <t>MAPX 205</t>
         </is>
       </c>
       <c r="D1084" s="2" t="inlineStr"/>
@@ -40391,7 +40391,7 @@
       </c>
       <c r="C1085" s="4" t="inlineStr">
         <is>
-          <t>MAPX-205</t>
+          <t>MAPX 205</t>
         </is>
       </c>
       <c r="D1085" s="4" t="inlineStr"/>
@@ -40426,7 +40426,7 @@
       </c>
       <c r="C1086" s="2" t="inlineStr">
         <is>
-          <t>MAPX-207</t>
+          <t>MAPX 207</t>
         </is>
       </c>
       <c r="D1086" s="2" t="inlineStr"/>
@@ -40461,7 +40461,7 @@
       </c>
       <c r="C1087" s="4" t="inlineStr">
         <is>
-          <t>MAPX-207</t>
+          <t>MAPX 207</t>
         </is>
       </c>
       <c r="D1087" s="4" t="inlineStr"/>
@@ -40496,7 +40496,7 @@
       </c>
       <c r="C1088" s="2" t="inlineStr">
         <is>
-          <t>MAPX-207</t>
+          <t>MAPX 207</t>
         </is>
       </c>
       <c r="D1088" s="2" t="inlineStr"/>
@@ -40531,7 +40531,7 @@
       </c>
       <c r="C1089" s="4" t="inlineStr">
         <is>
-          <t>MAPX-210</t>
+          <t>MAPX 210</t>
         </is>
       </c>
       <c r="D1089" s="4" t="inlineStr"/>
@@ -40566,7 +40566,7 @@
       </c>
       <c r="C1090" s="2" t="inlineStr">
         <is>
-          <t>MAPX-210</t>
+          <t>MAPX 210</t>
         </is>
       </c>
       <c r="D1090" s="2" t="inlineStr"/>
@@ -40601,7 +40601,7 @@
       </c>
       <c r="C1091" s="4" t="inlineStr">
         <is>
-          <t>MAPX-210</t>
+          <t>MAPX 210</t>
         </is>
       </c>
       <c r="D1091" s="4" t="inlineStr"/>
@@ -40636,7 +40636,7 @@
       </c>
       <c r="C1092" s="2" t="inlineStr">
         <is>
-          <t>MAPX-210</t>
+          <t>MAPX 210</t>
         </is>
       </c>
       <c r="D1092" s="2" t="inlineStr"/>
@@ -40671,7 +40671,7 @@
       </c>
       <c r="C1093" s="4" t="inlineStr">
         <is>
-          <t>MAPX-210</t>
+          <t>MAPX 210</t>
         </is>
       </c>
       <c r="D1093" s="4" t="inlineStr"/>
@@ -40706,7 +40706,7 @@
       </c>
       <c r="C1094" s="2" t="inlineStr">
         <is>
-          <t>MAPX-309</t>
+          <t>MAPX 309</t>
         </is>
       </c>
       <c r="D1094" s="2" t="inlineStr"/>
@@ -40741,7 +40741,7 @@
       </c>
       <c r="C1095" s="4" t="inlineStr">
         <is>
-          <t>MAPX-309</t>
+          <t>MAPX 309</t>
         </is>
       </c>
       <c r="D1095" s="4" t="inlineStr"/>
@@ -40776,7 +40776,7 @@
       </c>
       <c r="C1096" s="2" t="inlineStr">
         <is>
-          <t>MAPX-309</t>
+          <t>MAPX 309</t>
         </is>
       </c>
       <c r="D1096" s="2" t="inlineStr"/>
@@ -40811,7 +40811,7 @@
       </c>
       <c r="C1097" s="4" t="inlineStr">
         <is>
-          <t>MAPX-309</t>
+          <t>MAPX 309</t>
         </is>
       </c>
       <c r="D1097" s="4" t="inlineStr"/>
@@ -40846,7 +40846,7 @@
       </c>
       <c r="C1098" s="2" t="inlineStr">
         <is>
-          <t>MAPX-309</t>
+          <t>MAPX 309</t>
         </is>
       </c>
       <c r="D1098" s="2" t="inlineStr"/>
@@ -40881,7 +40881,7 @@
       </c>
       <c r="C1099" s="4" t="inlineStr">
         <is>
-          <t>MAPX-313</t>
+          <t>MAPX 313</t>
         </is>
       </c>
       <c r="D1099" s="4" t="inlineStr"/>
@@ -40916,7 +40916,7 @@
       </c>
       <c r="C1100" s="2" t="inlineStr">
         <is>
-          <t>MAPX-313</t>
+          <t>MAPX 313</t>
         </is>
       </c>
       <c r="D1100" s="2" t="inlineStr"/>
@@ -40951,7 +40951,7 @@
       </c>
       <c r="C1101" s="4" t="inlineStr">
         <is>
-          <t>MAPX-313</t>
+          <t>MAPX 313</t>
         </is>
       </c>
       <c r="D1101" s="4" t="inlineStr"/>
@@ -40986,7 +40986,7 @@
       </c>
       <c r="C1102" s="2" t="inlineStr">
         <is>
-          <t>MAPX-313</t>
+          <t>MAPX 313</t>
         </is>
       </c>
       <c r="D1102" s="2" t="inlineStr"/>
@@ -41021,7 +41021,7 @@
       </c>
       <c r="C1103" s="4" t="inlineStr">
         <is>
-          <t>MAPX-313</t>
+          <t>MAPX 313</t>
         </is>
       </c>
       <c r="D1103" s="4" t="inlineStr"/>
@@ -41056,7 +41056,7 @@
       </c>
       <c r="C1104" s="2" t="inlineStr">
         <is>
-          <t>MFPX-307</t>
+          <t>MFPX 307</t>
         </is>
       </c>
       <c r="D1104" s="2" t="inlineStr"/>
@@ -41091,7 +41091,7 @@
       </c>
       <c r="C1105" s="4" t="inlineStr">
         <is>
-          <t>MFPX-307</t>
+          <t>MFPX 307</t>
         </is>
       </c>
       <c r="D1105" s="4" t="inlineStr"/>
@@ -41126,7 +41126,7 @@
       </c>
       <c r="C1106" s="2" t="inlineStr">
         <is>
-          <t>MFPX-307</t>
+          <t>MFPX 307</t>
         </is>
       </c>
       <c r="D1106" s="2" t="inlineStr"/>
@@ -41161,7 +41161,7 @@
       </c>
       <c r="C1107" s="4" t="inlineStr">
         <is>
-          <t>MFPX-307</t>
+          <t>MFPX 307</t>
         </is>
       </c>
       <c r="D1107" s="4" t="inlineStr"/>
@@ -41196,7 +41196,7 @@
       </c>
       <c r="C1108" s="2" t="inlineStr">
         <is>
-          <t>MMB-304</t>
+          <t>MMB 304</t>
         </is>
       </c>
       <c r="D1108" s="2" t="inlineStr"/>
@@ -41231,7 +41231,7 @@
       </c>
       <c r="C1109" s="4" t="inlineStr">
         <is>
-          <t>MMB-304</t>
+          <t>MMB 304</t>
         </is>
       </c>
       <c r="D1109" s="4" t="inlineStr"/>
@@ -41266,7 +41266,7 @@
       </c>
       <c r="C1110" s="2" t="inlineStr">
         <is>
-          <t>MMB-304</t>
+          <t>MMB 304</t>
         </is>
       </c>
       <c r="D1110" s="2" t="inlineStr"/>
@@ -41301,7 +41301,7 @@
       </c>
       <c r="C1111" s="4" t="inlineStr">
         <is>
-          <t>MMB-304</t>
+          <t>MMB 304</t>
         </is>
       </c>
       <c r="D1111" s="4" t="inlineStr"/>
@@ -41336,7 +41336,7 @@
       </c>
       <c r="C1112" s="2" t="inlineStr">
         <is>
-          <t>MMB-305</t>
+          <t>MMB 305</t>
         </is>
       </c>
       <c r="D1112" s="2" t="inlineStr"/>
@@ -41371,7 +41371,7 @@
       </c>
       <c r="C1113" s="4" t="inlineStr">
         <is>
-          <t>MMB-305</t>
+          <t>MMB 305</t>
         </is>
       </c>
       <c r="D1113" s="4" t="inlineStr"/>
@@ -41406,7 +41406,7 @@
       </c>
       <c r="C1114" s="2" t="inlineStr">
         <is>
-          <t>MMB-305</t>
+          <t>MMB 305</t>
         </is>
       </c>
       <c r="D1114" s="2" t="inlineStr"/>
@@ -41441,7 +41441,7 @@
       </c>
       <c r="C1115" s="4" t="inlineStr">
         <is>
-          <t>MMB-305</t>
+          <t>MMB 305</t>
         </is>
       </c>
       <c r="D1115" s="4" t="inlineStr"/>
@@ -41476,7 +41476,7 @@
       </c>
       <c r="C1116" s="2" t="inlineStr">
         <is>
-          <t>MMPX-303</t>
+          <t>MMPX 303</t>
         </is>
       </c>
       <c r="D1116" s="2" t="inlineStr"/>
@@ -41511,7 +41511,7 @@
       </c>
       <c r="C1117" s="4" t="inlineStr">
         <is>
-          <t>MMPX-303</t>
+          <t>MMPX 303</t>
         </is>
       </c>
       <c r="D1117" s="4" t="inlineStr"/>
@@ -41546,7 +41546,7 @@
       </c>
       <c r="C1118" s="2" t="inlineStr">
         <is>
-          <t>MMPX-303</t>
+          <t>MMPX 303</t>
         </is>
       </c>
       <c r="D1118" s="2" t="inlineStr"/>
@@ -41581,7 +41581,7 @@
       </c>
       <c r="C1119" s="4" t="inlineStr">
         <is>
-          <t>MMPX-303</t>
+          <t>MMPX 303</t>
         </is>
       </c>
       <c r="D1119" s="4" t="inlineStr"/>
@@ -41616,7 +41616,7 @@
       </c>
       <c r="C1120" s="2" t="inlineStr">
         <is>
-          <t>MMPX-304</t>
+          <t>MMPX 304</t>
         </is>
       </c>
       <c r="D1120" s="2" t="inlineStr"/>
@@ -41651,7 +41651,7 @@
       </c>
       <c r="C1121" s="4" t="inlineStr">
         <is>
-          <t>MMPX-304</t>
+          <t>MMPX 304</t>
         </is>
       </c>
       <c r="D1121" s="4" t="inlineStr"/>
@@ -41686,7 +41686,7 @@
       </c>
       <c r="C1122" s="2" t="inlineStr">
         <is>
-          <t>MMPX-304</t>
+          <t>MMPX 304</t>
         </is>
       </c>
       <c r="D1122" s="2" t="inlineStr"/>
@@ -41721,7 +41721,7 @@
       </c>
       <c r="C1123" s="4" t="inlineStr">
         <is>
-          <t>MMPX-304</t>
+          <t>MMPX 304</t>
         </is>
       </c>
       <c r="D1123" s="4" t="inlineStr"/>
@@ -41756,7 +41756,7 @@
       </c>
       <c r="C1124" s="2" t="inlineStr">
         <is>
-          <t>MMPX-403</t>
+          <t>MMPX 403</t>
         </is>
       </c>
       <c r="D1124" s="2" t="inlineStr"/>
@@ -41791,7 +41791,7 @@
       </c>
       <c r="C1125" s="4" t="inlineStr">
         <is>
-          <t>MMPX-403</t>
+          <t>MMPX 403</t>
         </is>
       </c>
       <c r="D1125" s="4" t="inlineStr"/>
@@ -41826,7 +41826,7 @@
       </c>
       <c r="C1126" s="2" t="inlineStr">
         <is>
-          <t>MMPX-403</t>
+          <t>MMPX 403</t>
         </is>
       </c>
       <c r="D1126" s="2" t="inlineStr"/>
@@ -41861,7 +41861,7 @@
       </c>
       <c r="C1127" s="4" t="inlineStr">
         <is>
-          <t>MMPX-403</t>
+          <t>MMPX 403</t>
         </is>
       </c>
       <c r="D1127" s="4" t="inlineStr"/>
@@ -41896,7 +41896,7 @@
       </c>
       <c r="C1128" s="2" t="inlineStr">
         <is>
-          <t>MMPX-404</t>
+          <t>MMPX 404</t>
         </is>
       </c>
       <c r="D1128" s="2" t="inlineStr"/>
@@ -41931,7 +41931,7 @@
       </c>
       <c r="C1129" s="4" t="inlineStr">
         <is>
-          <t>MMPX-404</t>
+          <t>MMPX 404</t>
         </is>
       </c>
       <c r="D1129" s="4" t="inlineStr"/>
@@ -41966,7 +41966,7 @@
       </c>
       <c r="C1130" s="2" t="inlineStr">
         <is>
-          <t>MMPX-404</t>
+          <t>MMPX 404</t>
         </is>
       </c>
       <c r="D1130" s="2" t="inlineStr"/>
@@ -42001,7 +42001,7 @@
       </c>
       <c r="C1131" s="4" t="inlineStr">
         <is>
-          <t>MMPX-404</t>
+          <t>MMPX 404</t>
         </is>
       </c>
       <c r="D1131" s="4" t="inlineStr"/>
@@ -42036,7 +42036,7 @@
       </c>
       <c r="C1132" s="2" t="inlineStr">
         <is>
-          <t>MOPX-204</t>
+          <t>MOPX 204</t>
         </is>
       </c>
       <c r="D1132" s="2" t="inlineStr"/>
@@ -42071,7 +42071,7 @@
       </c>
       <c r="C1133" s="4" t="inlineStr">
         <is>
-          <t>MOPX-204</t>
+          <t>MOPX 204</t>
         </is>
       </c>
       <c r="D1133" s="4" t="inlineStr"/>
@@ -42106,7 +42106,7 @@
       </c>
       <c r="C1134" s="2" t="inlineStr">
         <is>
-          <t>MOPX-204</t>
+          <t>MOPX 204</t>
         </is>
       </c>
       <c r="D1134" s="2" t="inlineStr"/>
@@ -42141,7 +42141,7 @@
       </c>
       <c r="C1135" s="4" t="inlineStr">
         <is>
-          <t>MOPX-204</t>
+          <t>MOPX 204</t>
         </is>
       </c>
       <c r="D1135" s="4" t="inlineStr"/>
@@ -42176,7 +42176,7 @@
       </c>
       <c r="C1136" s="2" t="inlineStr">
         <is>
-          <t>MOPX-204</t>
+          <t>MOPX 204</t>
         </is>
       </c>
       <c r="D1136" s="2" t="inlineStr"/>
@@ -42211,7 +42211,7 @@
       </c>
       <c r="C1137" s="4" t="inlineStr">
         <is>
-          <t>MOPX-205</t>
+          <t>MOPX 205</t>
         </is>
       </c>
       <c r="D1137" s="4" t="inlineStr"/>
@@ -42246,7 +42246,7 @@
       </c>
       <c r="C1138" s="2" t="inlineStr">
         <is>
-          <t>MOPX-205</t>
+          <t>MOPX 205</t>
         </is>
       </c>
       <c r="D1138" s="2" t="inlineStr"/>
@@ -42281,7 +42281,7 @@
       </c>
       <c r="C1139" s="4" t="inlineStr">
         <is>
-          <t>MOPX-205</t>
+          <t>MOPX 205</t>
         </is>
       </c>
       <c r="D1139" s="4" t="inlineStr"/>
@@ -42316,7 +42316,7 @@
       </c>
       <c r="C1140" s="2" t="inlineStr">
         <is>
-          <t>MOPX-205</t>
+          <t>MOPX 205</t>
         </is>
       </c>
       <c r="D1140" s="2" t="inlineStr"/>
@@ -42351,7 +42351,7 @@
       </c>
       <c r="C1141" s="4" t="inlineStr">
         <is>
-          <t>MOPX-205</t>
+          <t>MOPX 205</t>
         </is>
       </c>
       <c r="D1141" s="4" t="inlineStr"/>
@@ -42386,7 +42386,7 @@
       </c>
       <c r="C1142" s="2" t="inlineStr">
         <is>
-          <t>MOPX-207</t>
+          <t>MOPX 207</t>
         </is>
       </c>
       <c r="D1142" s="2" t="inlineStr"/>
@@ -42421,7 +42421,7 @@
       </c>
       <c r="C1143" s="4" t="inlineStr">
         <is>
-          <t>MOPX-207</t>
+          <t>MOPX 207</t>
         </is>
       </c>
       <c r="D1143" s="4" t="inlineStr"/>
@@ -42456,7 +42456,7 @@
       </c>
       <c r="C1144" s="2" t="inlineStr">
         <is>
-          <t>MOPX-207</t>
+          <t>MOPX 207</t>
         </is>
       </c>
       <c r="D1144" s="2" t="inlineStr"/>
@@ -42491,7 +42491,7 @@
       </c>
       <c r="C1145" s="4" t="inlineStr">
         <is>
-          <t>MOPX-209</t>
+          <t>MOPX 209</t>
         </is>
       </c>
       <c r="D1145" s="4" t="inlineStr"/>
@@ -42526,7 +42526,7 @@
       </c>
       <c r="C1146" s="2" t="inlineStr">
         <is>
-          <t>MOPX-209</t>
+          <t>MOPX 209</t>
         </is>
       </c>
       <c r="D1146" s="2" t="inlineStr"/>
@@ -42561,7 +42561,7 @@
       </c>
       <c r="C1147" s="4" t="inlineStr">
         <is>
-          <t>MOPX-209</t>
+          <t>MOPX 209</t>
         </is>
       </c>
       <c r="D1147" s="4" t="inlineStr"/>
@@ -42596,7 +42596,7 @@
       </c>
       <c r="C1148" s="2" t="inlineStr">
         <is>
-          <t>MOPX-209</t>
+          <t>MOPX 209</t>
         </is>
       </c>
       <c r="D1148" s="2" t="inlineStr"/>
@@ -42631,7 +42631,7 @@
       </c>
       <c r="C1149" s="4" t="inlineStr">
         <is>
-          <t>MOPX-209</t>
+          <t>MOPX 209</t>
         </is>
       </c>
       <c r="D1149" s="4" t="inlineStr"/>
@@ -42666,7 +42666,7 @@
       </c>
       <c r="C1150" s="2" t="inlineStr">
         <is>
-          <t>MOPX-210</t>
+          <t>MOPX 210</t>
         </is>
       </c>
       <c r="D1150" s="2" t="inlineStr"/>
@@ -42701,7 +42701,7 @@
       </c>
       <c r="C1151" s="4" t="inlineStr">
         <is>
-          <t>MOPX-210</t>
+          <t>MOPX 210</t>
         </is>
       </c>
       <c r="D1151" s="4" t="inlineStr"/>
@@ -42736,7 +42736,7 @@
       </c>
       <c r="C1152" s="2" t="inlineStr">
         <is>
-          <t>MOPX-210</t>
+          <t>MOPX 210</t>
         </is>
       </c>
       <c r="D1152" s="2" t="inlineStr"/>
@@ -42771,7 +42771,7 @@
       </c>
       <c r="C1153" s="4" t="inlineStr">
         <is>
-          <t>MOPX-210</t>
+          <t>MOPX 210</t>
         </is>
       </c>
       <c r="D1153" s="4" t="inlineStr"/>
@@ -42806,7 +42806,7 @@
       </c>
       <c r="C1154" s="2" t="inlineStr">
         <is>
-          <t>MOPX-210</t>
+          <t>MOPX 210</t>
         </is>
       </c>
       <c r="D1154" s="2" t="inlineStr"/>
@@ -42841,7 +42841,7 @@
       </c>
       <c r="C1155" s="4" t="inlineStr">
         <is>
-          <t>MOPX-213</t>
+          <t>MOPX 213</t>
         </is>
       </c>
       <c r="D1155" s="4" t="inlineStr"/>
@@ -42876,7 +42876,7 @@
       </c>
       <c r="C1156" s="2" t="inlineStr">
         <is>
-          <t>MOPX-213</t>
+          <t>MOPX 213</t>
         </is>
       </c>
       <c r="D1156" s="2" t="inlineStr"/>
@@ -42911,7 +42911,7 @@
       </c>
       <c r="C1157" s="4" t="inlineStr">
         <is>
-          <t>MOPX-213</t>
+          <t>MOPX 213</t>
         </is>
       </c>
       <c r="D1157" s="4" t="inlineStr"/>
@@ -42946,7 +42946,7 @@
       </c>
       <c r="C1158" s="2" t="inlineStr">
         <is>
-          <t>MOPX-213</t>
+          <t>MOPX 213</t>
         </is>
       </c>
       <c r="D1158" s="2" t="inlineStr"/>
@@ -42981,7 +42981,7 @@
       </c>
       <c r="C1159" s="4" t="inlineStr">
         <is>
-          <t>MOPX-213</t>
+          <t>MOPX 213</t>
         </is>
       </c>
       <c r="D1159" s="4" t="inlineStr"/>
@@ -43016,7 +43016,7 @@
       </c>
       <c r="C1160" s="2" t="inlineStr">
         <is>
-          <t>MOPX-309</t>
+          <t>MOPX 309</t>
         </is>
       </c>
       <c r="D1160" s="2" t="inlineStr"/>
@@ -43051,7 +43051,7 @@
       </c>
       <c r="C1161" s="4" t="inlineStr">
         <is>
-          <t>MOPX-309</t>
+          <t>MOPX 309</t>
         </is>
       </c>
       <c r="D1161" s="4" t="inlineStr"/>
@@ -43086,7 +43086,7 @@
       </c>
       <c r="C1162" s="2" t="inlineStr">
         <is>
-          <t>MOPX-309</t>
+          <t>MOPX 309</t>
         </is>
       </c>
       <c r="D1162" s="2" t="inlineStr"/>
@@ -43121,7 +43121,7 @@
       </c>
       <c r="C1163" s="4" t="inlineStr">
         <is>
-          <t>MOPX-309</t>
+          <t>MOPX 309</t>
         </is>
       </c>
       <c r="D1163" s="4" t="inlineStr"/>
@@ -43156,7 +43156,7 @@
       </c>
       <c r="C1164" s="2" t="inlineStr">
         <is>
-          <t>MOPX-309</t>
+          <t>MOPX 309</t>
         </is>
       </c>
       <c r="D1164" s="2" t="inlineStr"/>
@@ -43191,7 +43191,7 @@
       </c>
       <c r="C1165" s="4" t="inlineStr">
         <is>
-          <t>MOPX-310</t>
+          <t>MOPX 310</t>
         </is>
       </c>
       <c r="D1165" s="4" t="inlineStr"/>
@@ -43226,7 +43226,7 @@
       </c>
       <c r="C1166" s="2" t="inlineStr">
         <is>
-          <t>MOPX-310</t>
+          <t>MOPX 310</t>
         </is>
       </c>
       <c r="D1166" s="2" t="inlineStr"/>
@@ -43261,7 +43261,7 @@
       </c>
       <c r="C1167" s="4" t="inlineStr">
         <is>
-          <t>MOPX-310</t>
+          <t>MOPX 310</t>
         </is>
       </c>
       <c r="D1167" s="4" t="inlineStr"/>
@@ -43296,7 +43296,7 @@
       </c>
       <c r="C1168" s="2" t="inlineStr">
         <is>
-          <t>MOPX-310</t>
+          <t>MOPX 310</t>
         </is>
       </c>
       <c r="D1168" s="2" t="inlineStr"/>
@@ -43331,7 +43331,7 @@
       </c>
       <c r="C1169" s="4" t="inlineStr">
         <is>
-          <t>MOPX-310</t>
+          <t>MOPX 310</t>
         </is>
       </c>
       <c r="D1169" s="4" t="inlineStr"/>
@@ -43366,7 +43366,7 @@
       </c>
       <c r="C1170" s="2" t="inlineStr">
         <is>
-          <t>MOPX-313</t>
+          <t>MOPX 313</t>
         </is>
       </c>
       <c r="D1170" s="2" t="inlineStr"/>
@@ -43401,7 +43401,7 @@
       </c>
       <c r="C1171" s="4" t="inlineStr">
         <is>
-          <t>MOPX-313</t>
+          <t>MOPX 313</t>
         </is>
       </c>
       <c r="D1171" s="4" t="inlineStr"/>
@@ -43436,7 +43436,7 @@
       </c>
       <c r="C1172" s="2" t="inlineStr">
         <is>
-          <t>MOPX-313</t>
+          <t>MOPX 313</t>
         </is>
       </c>
       <c r="D1172" s="2" t="inlineStr"/>
@@ -43471,7 +43471,7 @@
       </c>
       <c r="C1173" s="4" t="inlineStr">
         <is>
-          <t>MOPX-313</t>
+          <t>MOPX 313</t>
         </is>
       </c>
       <c r="D1173" s="4" t="inlineStr"/>
@@ -43506,7 +43506,7 @@
       </c>
       <c r="C1174" s="2" t="inlineStr">
         <is>
-          <t>MOPX-313</t>
+          <t>MOPX 313</t>
         </is>
       </c>
       <c r="D1174" s="2" t="inlineStr"/>
@@ -43541,7 +43541,7 @@
       </c>
       <c r="C1175" s="4" t="inlineStr">
         <is>
-          <t>MSPX-303</t>
+          <t>MSPX 303</t>
         </is>
       </c>
       <c r="D1175" s="4" t="inlineStr"/>
@@ -43576,7 +43576,7 @@
       </c>
       <c r="C1176" s="2" t="inlineStr">
         <is>
-          <t>MSPX-303</t>
+          <t>MSPX 303</t>
         </is>
       </c>
       <c r="D1176" s="2" t="inlineStr"/>
@@ -43611,7 +43611,7 @@
       </c>
       <c r="C1177" s="4" t="inlineStr">
         <is>
-          <t>MSPX-303</t>
+          <t>MSPX 303</t>
         </is>
       </c>
       <c r="D1177" s="4" t="inlineStr"/>
@@ -43646,7 +43646,7 @@
       </c>
       <c r="C1178" s="2" t="inlineStr">
         <is>
-          <t>MSPX-303</t>
+          <t>MSPX 303</t>
         </is>
       </c>
       <c r="D1178" s="2" t="inlineStr"/>
@@ -43681,7 +43681,7 @@
       </c>
       <c r="C1179" s="4" t="inlineStr">
         <is>
-          <t>MSPX-403</t>
+          <t>MSPX 403</t>
         </is>
       </c>
       <c r="D1179" s="4" t="inlineStr"/>
@@ -43716,7 +43716,7 @@
       </c>
       <c r="C1180" s="2" t="inlineStr">
         <is>
-          <t>MSPX-403</t>
+          <t>MSPX 403</t>
         </is>
       </c>
       <c r="D1180" s="2" t="inlineStr"/>
@@ -43751,7 +43751,7 @@
       </c>
       <c r="C1181" s="4" t="inlineStr">
         <is>
-          <t>MSPX-403</t>
+          <t>MSPX 403</t>
         </is>
       </c>
       <c r="D1181" s="4" t="inlineStr"/>
@@ -43786,7 +43786,7 @@
       </c>
       <c r="C1182" s="2" t="inlineStr">
         <is>
-          <t>MSPX-403</t>
+          <t>MSPX 403</t>
         </is>
       </c>
       <c r="D1182" s="2" t="inlineStr"/>
@@ -43821,7 +43821,7 @@
       </c>
       <c r="C1183" s="4" t="inlineStr">
         <is>
-          <t>PA-600</t>
+          <t>PA 600</t>
         </is>
       </c>
       <c r="D1183" s="4" t="inlineStr"/>
@@ -43856,7 +43856,7 @@
       </c>
       <c r="C1184" s="2" t="inlineStr">
         <is>
-          <t>PA-600</t>
+          <t>PA 600</t>
         </is>
       </c>
       <c r="D1184" s="2" t="inlineStr"/>
@@ -43891,7 +43891,7 @@
       </c>
       <c r="C1185" s="4" t="inlineStr">
         <is>
-          <t>PA-600</t>
+          <t>PA 600</t>
         </is>
       </c>
       <c r="D1185" s="4" t="inlineStr"/>
@@ -43926,7 +43926,7 @@
       </c>
       <c r="C1186" s="2" t="inlineStr">
         <is>
-          <t>PA-600</t>
+          <t>PA 600</t>
         </is>
       </c>
       <c r="D1186" s="2" t="inlineStr"/>
@@ -43961,7 +43961,7 @@
       </c>
       <c r="C1187" s="4" t="inlineStr">
         <is>
-          <t>PA-605</t>
+          <t>PA 605</t>
         </is>
       </c>
       <c r="D1187" s="4" t="inlineStr"/>
@@ -43996,7 +43996,7 @@
       </c>
       <c r="C1188" s="2" t="inlineStr">
         <is>
-          <t>PA-605</t>
+          <t>PA 605</t>
         </is>
       </c>
       <c r="D1188" s="2" t="inlineStr"/>
@@ -44031,7 +44031,7 @@
       </c>
       <c r="C1189" s="4" t="inlineStr">
         <is>
-          <t>PA-605</t>
+          <t>PA 605</t>
         </is>
       </c>
       <c r="D1189" s="4" t="inlineStr"/>
@@ -44066,7 +44066,7 @@
       </c>
       <c r="C1190" s="2" t="inlineStr">
         <is>
-          <t>PA-605</t>
+          <t>PA 605</t>
         </is>
       </c>
       <c r="D1190" s="2" t="inlineStr"/>
@@ -44101,7 +44101,7 @@
       </c>
       <c r="C1191" s="4" t="inlineStr">
         <is>
-          <t>PA-610</t>
+          <t>PA 610</t>
         </is>
       </c>
       <c r="D1191" s="4" t="inlineStr"/>
@@ -44136,7 +44136,7 @@
       </c>
       <c r="C1192" s="2" t="inlineStr">
         <is>
-          <t>PA-610</t>
+          <t>PA 610</t>
         </is>
       </c>
       <c r="D1192" s="2" t="inlineStr"/>
@@ -44171,7 +44171,7 @@
       </c>
       <c r="C1193" s="4" t="inlineStr">
         <is>
-          <t>PA-610</t>
+          <t>PA 610</t>
         </is>
       </c>
       <c r="D1193" s="4" t="inlineStr"/>
@@ -44206,7 +44206,7 @@
       </c>
       <c r="C1194" s="2" t="inlineStr">
         <is>
-          <t>PA-610</t>
+          <t>PA 610</t>
         </is>
       </c>
       <c r="D1194" s="2" t="inlineStr"/>
@@ -44241,7 +44241,7 @@
       </c>
       <c r="C1195" s="4" t="inlineStr">
         <is>
-          <t>PA-615</t>
+          <t>PA 615</t>
         </is>
       </c>
       <c r="D1195" s="4" t="inlineStr"/>
@@ -44276,7 +44276,7 @@
       </c>
       <c r="C1196" s="2" t="inlineStr">
         <is>
-          <t>PA-615</t>
+          <t>PA 615</t>
         </is>
       </c>
       <c r="D1196" s="2" t="inlineStr"/>
@@ -44311,7 +44311,7 @@
       </c>
       <c r="C1197" s="4" t="inlineStr">
         <is>
-          <t>PA-615</t>
+          <t>PA 615</t>
         </is>
       </c>
       <c r="D1197" s="4" t="inlineStr"/>
@@ -44346,7 +44346,7 @@
       </c>
       <c r="C1198" s="2" t="inlineStr">
         <is>
-          <t>PA-615</t>
+          <t>PA 615</t>
         </is>
       </c>
       <c r="D1198" s="2" t="inlineStr"/>
@@ -44381,7 +44381,7 @@
       </c>
       <c r="C1199" s="4" t="inlineStr">
         <is>
-          <t>PA-625</t>
+          <t>PA 625</t>
         </is>
       </c>
       <c r="D1199" s="4" t="inlineStr">
@@ -44420,7 +44420,7 @@
       </c>
       <c r="C1200" s="2" t="inlineStr">
         <is>
-          <t>PA-625</t>
+          <t>PA 625</t>
         </is>
       </c>
       <c r="D1200" s="2" t="inlineStr">
@@ -44459,7 +44459,7 @@
       </c>
       <c r="C1201" s="4" t="inlineStr">
         <is>
-          <t>PA-635</t>
+          <t>PA 635</t>
         </is>
       </c>
       <c r="D1201" s="4" t="inlineStr">
@@ -44498,7 +44498,7 @@
       </c>
       <c r="C1202" s="2" t="inlineStr">
         <is>
-          <t>PA-635</t>
+          <t>PA 635</t>
         </is>
       </c>
       <c r="D1202" s="2" t="inlineStr">
@@ -44537,7 +44537,7 @@
       </c>
       <c r="C1203" s="4" t="inlineStr">
         <is>
-          <t>PU-100</t>
+          <t>PU 100</t>
         </is>
       </c>
       <c r="D1203" s="4" t="inlineStr"/>
@@ -44572,7 +44572,7 @@
       </c>
       <c r="C1204" s="2" t="inlineStr">
         <is>
-          <t>PU-100</t>
+          <t>PU 100</t>
         </is>
       </c>
       <c r="D1204" s="2" t="inlineStr"/>
@@ -44607,7 +44607,7 @@
       </c>
       <c r="C1205" s="4" t="inlineStr">
         <is>
-          <t>PU-100</t>
+          <t>PU 100</t>
         </is>
       </c>
       <c r="D1205" s="4" t="inlineStr"/>
@@ -44642,7 +44642,7 @@
       </c>
       <c r="C1206" s="2" t="inlineStr">
         <is>
-          <t>PU-100</t>
+          <t>PU 100</t>
         </is>
       </c>
       <c r="D1206" s="2" t="inlineStr"/>
@@ -44677,7 +44677,7 @@
       </c>
       <c r="C1207" s="4" t="inlineStr">
         <is>
-          <t>PU-150</t>
+          <t>PU 150</t>
         </is>
       </c>
       <c r="D1207" s="4" t="inlineStr"/>
@@ -44712,7 +44712,7 @@
       </c>
       <c r="C1208" s="2" t="inlineStr">
         <is>
-          <t>PU-150</t>
+          <t>PU 150</t>
         </is>
       </c>
       <c r="D1208" s="2" t="inlineStr"/>
@@ -44747,7 +44747,7 @@
       </c>
       <c r="C1209" s="4" t="inlineStr">
         <is>
-          <t>PU-150</t>
+          <t>PU 150</t>
         </is>
       </c>
       <c r="D1209" s="4" t="inlineStr"/>
@@ -44782,7 +44782,7 @@
       </c>
       <c r="C1210" s="2" t="inlineStr">
         <is>
-          <t>PU-150</t>
+          <t>PU 150</t>
         </is>
       </c>
       <c r="D1210" s="2" t="inlineStr"/>
@@ -44817,7 +44817,7 @@
       </c>
       <c r="C1211" s="4" t="inlineStr">
         <is>
-          <t>S-300</t>
+          <t>S 300</t>
         </is>
       </c>
       <c r="D1211" s="4" t="inlineStr">
@@ -44856,7 +44856,7 @@
       </c>
       <c r="C1212" s="2" t="inlineStr">
         <is>
-          <t>S-300</t>
+          <t>S 300</t>
         </is>
       </c>
       <c r="D1212" s="2" t="inlineStr">
@@ -44895,7 +44895,7 @@
       </c>
       <c r="C1213" s="4" t="inlineStr">
         <is>
-          <t>S-300</t>
+          <t>S 300</t>
         </is>
       </c>
       <c r="D1213" s="4" t="inlineStr">
@@ -44934,7 +44934,7 @@
       </c>
       <c r="C1214" s="2" t="inlineStr">
         <is>
-          <t>S-500</t>
+          <t>S 500</t>
         </is>
       </c>
       <c r="D1214" s="2" t="inlineStr">
@@ -44973,7 +44973,7 @@
       </c>
       <c r="C1215" s="4" t="inlineStr">
         <is>
-          <t>S-500</t>
+          <t>S 500</t>
         </is>
       </c>
       <c r="D1215" s="4" t="inlineStr">
@@ -45012,7 +45012,7 @@
       </c>
       <c r="C1216" s="2" t="inlineStr">
         <is>
-          <t>S-500</t>
+          <t>S 500</t>
         </is>
       </c>
       <c r="D1216" s="2" t="inlineStr">
@@ -45051,7 +45051,7 @@
       </c>
       <c r="C1217" s="4" t="inlineStr">
         <is>
-          <t>S-811</t>
+          <t>S 811</t>
         </is>
       </c>
       <c r="D1217" s="4" t="inlineStr">
@@ -45090,7 +45090,7 @@
       </c>
       <c r="C1218" s="2" t="inlineStr">
         <is>
-          <t>S-811</t>
+          <t>S 811</t>
         </is>
       </c>
       <c r="D1218" s="2" t="inlineStr">
@@ -45129,7 +45129,7 @@
       </c>
       <c r="C1219" s="4" t="inlineStr">
         <is>
-          <t>S-816</t>
+          <t>S 816</t>
         </is>
       </c>
       <c r="D1219" s="4" t="inlineStr">
@@ -45168,7 +45168,7 @@
       </c>
       <c r="C1220" s="2" t="inlineStr">
         <is>
-          <t>S-816</t>
+          <t>S 816</t>
         </is>
       </c>
       <c r="D1220" s="2" t="inlineStr">
@@ -45207,7 +45207,7 @@
       </c>
       <c r="C1221" s="4" t="inlineStr">
         <is>
-          <t>S-820</t>
+          <t>S 820</t>
         </is>
       </c>
       <c r="D1221" s="4" t="inlineStr">
@@ -45246,7 +45246,7 @@
       </c>
       <c r="C1222" s="2" t="inlineStr">
         <is>
-          <t>S-820</t>
+          <t>S 820</t>
         </is>
       </c>
       <c r="D1222" s="2" t="inlineStr">
@@ -45285,7 +45285,7 @@
       </c>
       <c r="C1223" s="4" t="inlineStr">
         <is>
-          <t>S-821</t>
+          <t>S 821</t>
         </is>
       </c>
       <c r="D1223" s="4" t="inlineStr">
@@ -45324,7 +45324,7 @@
       </c>
       <c r="C1224" s="2" t="inlineStr">
         <is>
-          <t>S-821</t>
+          <t>S 821</t>
         </is>
       </c>
       <c r="D1224" s="2" t="inlineStr">
@@ -45363,7 +45363,7 @@
       </c>
       <c r="C1225" s="4" t="inlineStr">
         <is>
-          <t>S-825</t>
+          <t>S 825</t>
         </is>
       </c>
       <c r="D1225" s="4" t="inlineStr">
@@ -45402,7 +45402,7 @@
       </c>
       <c r="C1226" s="2" t="inlineStr">
         <is>
-          <t>S-825</t>
+          <t>S 825</t>
         </is>
       </c>
       <c r="D1226" s="2" t="inlineStr">
@@ -45441,7 +45441,7 @@
       </c>
       <c r="C1227" s="4" t="inlineStr">
         <is>
-          <t>S-826</t>
+          <t>S 826</t>
         </is>
       </c>
       <c r="D1227" s="4" t="inlineStr">
@@ -45480,7 +45480,7 @@
       </c>
       <c r="C1228" s="2" t="inlineStr">
         <is>
-          <t>S-826</t>
+          <t>S 826</t>
         </is>
       </c>
       <c r="D1228" s="2" t="inlineStr">
@@ -45519,7 +45519,7 @@
       </c>
       <c r="C1229" s="4" t="inlineStr">
         <is>
-          <t>S-830</t>
+          <t>S 830</t>
         </is>
       </c>
       <c r="D1229" s="4" t="inlineStr">
@@ -45558,7 +45558,7 @@
       </c>
       <c r="C1230" s="2" t="inlineStr">
         <is>
-          <t>S-830</t>
+          <t>S 830</t>
         </is>
       </c>
       <c r="D1230" s="2" t="inlineStr">
@@ -45597,7 +45597,7 @@
       </c>
       <c r="C1231" s="4" t="inlineStr">
         <is>
-          <t>S-831</t>
+          <t>S 831</t>
         </is>
       </c>
       <c r="D1231" s="4" t="inlineStr">
@@ -45636,7 +45636,7 @@
       </c>
       <c r="C1232" s="2" t="inlineStr">
         <is>
-          <t>S-831</t>
+          <t>S 831</t>
         </is>
       </c>
       <c r="D1232" s="2" t="inlineStr">
@@ -45675,7 +45675,7 @@
       </c>
       <c r="C1233" s="4" t="inlineStr">
         <is>
-          <t>S-835</t>
+          <t>S 835</t>
         </is>
       </c>
       <c r="D1233" s="4" t="inlineStr">
@@ -45714,7 +45714,7 @@
       </c>
       <c r="C1234" s="2" t="inlineStr">
         <is>
-          <t>S-835</t>
+          <t>S 835</t>
         </is>
       </c>
       <c r="D1234" s="2" t="inlineStr">
@@ -45753,7 +45753,7 @@
       </c>
       <c r="C1235" s="4" t="inlineStr">
         <is>
-          <t>S-836</t>
+          <t>S 836</t>
         </is>
       </c>
       <c r="D1235" s="4" t="inlineStr">
@@ -45792,7 +45792,7 @@
       </c>
       <c r="C1236" s="2" t="inlineStr">
         <is>
-          <t>S-836</t>
+          <t>S 836</t>
         </is>
       </c>
       <c r="D1236" s="2" t="inlineStr">
@@ -45831,7 +45831,7 @@
       </c>
       <c r="C1237" s="4" t="inlineStr">
         <is>
-          <t>S-840</t>
+          <t>S 840</t>
         </is>
       </c>
       <c r="D1237" s="4" t="inlineStr">
@@ -45870,7 +45870,7 @@
       </c>
       <c r="C1238" s="2" t="inlineStr">
         <is>
-          <t>S-840</t>
+          <t>S 840</t>
         </is>
       </c>
       <c r="D1238" s="2" t="inlineStr">
@@ -45909,7 +45909,7 @@
       </c>
       <c r="C1239" s="4" t="inlineStr">
         <is>
-          <t>S-841</t>
+          <t>S 841</t>
         </is>
       </c>
       <c r="D1239" s="4" t="inlineStr">
@@ -45948,7 +45948,7 @@
       </c>
       <c r="C1240" s="2" t="inlineStr">
         <is>
-          <t>S-841</t>
+          <t>S 841</t>
         </is>
       </c>
       <c r="D1240" s="2" t="inlineStr">
@@ -45987,7 +45987,7 @@
       </c>
       <c r="C1241" s="4" t="inlineStr">
         <is>
-          <t>S-845</t>
+          <t>S 845</t>
         </is>
       </c>
       <c r="D1241" s="4" t="inlineStr">
@@ -46026,7 +46026,7 @@
       </c>
       <c r="C1242" s="2" t="inlineStr">
         <is>
-          <t>S-845</t>
+          <t>S 845</t>
         </is>
       </c>
       <c r="D1242" s="2" t="inlineStr">
@@ -46065,7 +46065,7 @@
       </c>
       <c r="C1243" s="4" t="inlineStr">
         <is>
-          <t>S-846</t>
+          <t>S 846</t>
         </is>
       </c>
       <c r="D1243" s="4" t="inlineStr">
@@ -46104,7 +46104,7 @@
       </c>
       <c r="C1244" s="2" t="inlineStr">
         <is>
-          <t>S-846</t>
+          <t>S 846</t>
         </is>
       </c>
       <c r="D1244" s="2" t="inlineStr">
@@ -46143,7 +46143,7 @@
       </c>
       <c r="C1245" s="4" t="inlineStr">
         <is>
-          <t>S-850</t>
+          <t>S 850</t>
         </is>
       </c>
       <c r="D1245" s="4" t="inlineStr">
@@ -46182,7 +46182,7 @@
       </c>
       <c r="C1246" s="2" t="inlineStr">
         <is>
-          <t>S-850</t>
+          <t>S 850</t>
         </is>
       </c>
       <c r="D1246" s="2" t="inlineStr">
@@ -46221,7 +46221,7 @@
       </c>
       <c r="C1247" s="4" t="inlineStr">
         <is>
-          <t>S-851</t>
+          <t>S 851</t>
         </is>
       </c>
       <c r="D1247" s="4" t="inlineStr">
@@ -46260,7 +46260,7 @@
       </c>
       <c r="C1248" s="2" t="inlineStr">
         <is>
-          <t>S-851</t>
+          <t>S 851</t>
         </is>
       </c>
       <c r="D1248" s="2" t="inlineStr">
@@ -46299,7 +46299,7 @@
       </c>
       <c r="C1249" s="4" t="inlineStr">
         <is>
-          <t>S-855</t>
+          <t>S 855</t>
         </is>
       </c>
       <c r="D1249" s="4" t="inlineStr">
@@ -46338,7 +46338,7 @@
       </c>
       <c r="C1250" s="2" t="inlineStr">
         <is>
-          <t>S-855</t>
+          <t>S 855</t>
         </is>
       </c>
       <c r="D1250" s="2" t="inlineStr">
@@ -46377,7 +46377,7 @@
       </c>
       <c r="C1251" s="4" t="inlineStr">
         <is>
-          <t>S-856</t>
+          <t>S 856</t>
         </is>
       </c>
       <c r="D1251" s="4" t="inlineStr">
@@ -46416,7 +46416,7 @@
       </c>
       <c r="C1252" s="2" t="inlineStr">
         <is>
-          <t>S-856</t>
+          <t>S 856</t>
         </is>
       </c>
       <c r="D1252" s="2" t="inlineStr">
@@ -46455,7 +46455,7 @@
       </c>
       <c r="C1253" s="4" t="inlineStr">
         <is>
-          <t>S-860</t>
+          <t>S 860</t>
         </is>
       </c>
       <c r="D1253" s="4" t="inlineStr">
@@ -46494,7 +46494,7 @@
       </c>
       <c r="C1254" s="2" t="inlineStr">
         <is>
-          <t>S-860</t>
+          <t>S 860</t>
         </is>
       </c>
       <c r="D1254" s="2" t="inlineStr">
@@ -46533,7 +46533,7 @@
       </c>
       <c r="C1255" s="4" t="inlineStr">
         <is>
-          <t>S-861</t>
+          <t>S 861</t>
         </is>
       </c>
       <c r="D1255" s="4" t="inlineStr">
@@ -46572,7 +46572,7 @@
       </c>
       <c r="C1256" s="2" t="inlineStr">
         <is>
-          <t>S-861</t>
+          <t>S 861</t>
         </is>
       </c>
       <c r="D1256" s="2" t="inlineStr">
@@ -46611,7 +46611,7 @@
       </c>
       <c r="C1257" s="4" t="inlineStr">
         <is>
-          <t>S-865</t>
+          <t>S 865</t>
         </is>
       </c>
       <c r="D1257" s="4" t="inlineStr">
@@ -46650,7 +46650,7 @@
       </c>
       <c r="C1258" s="2" t="inlineStr">
         <is>
-          <t>S-865</t>
+          <t>S 865</t>
         </is>
       </c>
       <c r="D1258" s="2" t="inlineStr">
@@ -46689,7 +46689,7 @@
       </c>
       <c r="C1259" s="4" t="inlineStr">
         <is>
-          <t>S-866</t>
+          <t>S 866</t>
         </is>
       </c>
       <c r="D1259" s="4" t="inlineStr">
@@ -46728,7 +46728,7 @@
       </c>
       <c r="C1260" s="2" t="inlineStr">
         <is>
-          <t>S-866</t>
+          <t>S 866</t>
         </is>
       </c>
       <c r="D1260" s="2" t="inlineStr">
@@ -46767,7 +46767,7 @@
       </c>
       <c r="C1261" s="4" t="inlineStr">
         <is>
-          <t>S-870</t>
+          <t>S 870</t>
         </is>
       </c>
       <c r="D1261" s="4" t="inlineStr">
@@ -46806,7 +46806,7 @@
       </c>
       <c r="C1262" s="2" t="inlineStr">
         <is>
-          <t>S-870</t>
+          <t>S 870</t>
         </is>
       </c>
       <c r="D1262" s="2" t="inlineStr">
@@ -46845,7 +46845,7 @@
       </c>
       <c r="C1263" s="4" t="inlineStr">
         <is>
-          <t>S-871</t>
+          <t>S 871</t>
         </is>
       </c>
       <c r="D1263" s="4" t="inlineStr">
@@ -46884,7 +46884,7 @@
       </c>
       <c r="C1264" s="2" t="inlineStr">
         <is>
-          <t>S-871</t>
+          <t>S 871</t>
         </is>
       </c>
       <c r="D1264" s="2" t="inlineStr">
@@ -46923,7 +46923,7 @@
       </c>
       <c r="C1265" s="4" t="inlineStr">
         <is>
-          <t>S-875</t>
+          <t>S 875</t>
         </is>
       </c>
       <c r="D1265" s="4" t="inlineStr">
@@ -46962,7 +46962,7 @@
       </c>
       <c r="C1266" s="2" t="inlineStr">
         <is>
-          <t>S-875</t>
+          <t>S 875</t>
         </is>
       </c>
       <c r="D1266" s="2" t="inlineStr">
@@ -47001,7 +47001,7 @@
       </c>
       <c r="C1267" s="4" t="inlineStr">
         <is>
-          <t>S-876</t>
+          <t>S 876</t>
         </is>
       </c>
       <c r="D1267" s="4" t="inlineStr">
@@ -47040,7 +47040,7 @@
       </c>
       <c r="C1268" s="2" t="inlineStr">
         <is>
-          <t>S-876</t>
+          <t>S 876</t>
         </is>
       </c>
       <c r="D1268" s="2" t="inlineStr">
@@ -47079,7 +47079,7 @@
       </c>
       <c r="C1269" s="4" t="inlineStr">
         <is>
-          <t>S-880</t>
+          <t>S 880</t>
         </is>
       </c>
       <c r="D1269" s="4" t="inlineStr">
@@ -47118,7 +47118,7 @@
       </c>
       <c r="C1270" s="2" t="inlineStr">
         <is>
-          <t>S-880</t>
+          <t>S 880</t>
         </is>
       </c>
       <c r="D1270" s="2" t="inlineStr">
@@ -47157,7 +47157,7 @@
       </c>
       <c r="C1271" s="4" t="inlineStr">
         <is>
-          <t>S-881</t>
+          <t>S 881</t>
         </is>
       </c>
       <c r="D1271" s="4" t="inlineStr">
@@ -47196,7 +47196,7 @@
       </c>
       <c r="C1272" s="2" t="inlineStr">
         <is>
-          <t>S-881</t>
+          <t>S 881</t>
         </is>
       </c>
       <c r="D1272" s="2" t="inlineStr">
@@ -47235,7 +47235,7 @@
       </c>
       <c r="C1273" s="4" t="inlineStr">
         <is>
-          <t>S-885</t>
+          <t>S 885</t>
         </is>
       </c>
       <c r="D1273" s="4" t="inlineStr">
@@ -47274,7 +47274,7 @@
       </c>
       <c r="C1274" s="2" t="inlineStr">
         <is>
-          <t>S-885</t>
+          <t>S 885</t>
         </is>
       </c>
       <c r="D1274" s="2" t="inlineStr">
@@ -47313,7 +47313,7 @@
       </c>
       <c r="C1275" s="4" t="inlineStr">
         <is>
-          <t>S-886</t>
+          <t>S 886</t>
         </is>
       </c>
       <c r="D1275" s="4" t="inlineStr">
@@ -47352,7 +47352,7 @@
       </c>
       <c r="C1276" s="2" t="inlineStr">
         <is>
-          <t>S-886</t>
+          <t>S 886</t>
         </is>
       </c>
       <c r="D1276" s="2" t="inlineStr">
@@ -47391,7 +47391,7 @@
       </c>
       <c r="C1277" s="4" t="inlineStr">
         <is>
-          <t>WHPX-405</t>
+          <t>WHPX 405</t>
         </is>
       </c>
       <c r="D1277" s="4" t="inlineStr"/>
@@ -47426,7 +47426,7 @@
       </c>
       <c r="C1278" s="2" t="inlineStr">
         <is>
-          <t>WHPX-405</t>
+          <t>WHPX 405</t>
         </is>
       </c>
       <c r="D1278" s="2" t="inlineStr"/>
@@ -47461,7 +47461,7 @@
       </c>
       <c r="C1279" s="4" t="inlineStr">
         <is>
-          <t>WHPX-405</t>
+          <t>WHPX 405</t>
         </is>
       </c>
       <c r="D1279" s="4" t="inlineStr"/>
@@ -47496,7 +47496,7 @@
       </c>
       <c r="C1280" s="2" t="inlineStr">
         <is>
-          <t>WHPX-405</t>
+          <t>WHPX 405</t>
         </is>
       </c>
       <c r="D1280" s="2" t="inlineStr"/>
@@ -47531,7 +47531,7 @@
       </c>
       <c r="C1281" s="4" t="inlineStr">
         <is>
-          <t>WHPX-405</t>
+          <t>WHPX 405</t>
         </is>
       </c>
       <c r="D1281" s="4" t="inlineStr"/>
@@ -47566,7 +47566,7 @@
       </c>
       <c r="C1282" s="2" t="inlineStr">
         <is>
-          <t>WHPX-505</t>
+          <t>WHPX 505</t>
         </is>
       </c>
       <c r="D1282" s="2" t="inlineStr"/>
@@ -47601,7 +47601,7 @@
       </c>
       <c r="C1283" s="4" t="inlineStr">
         <is>
-          <t>WHPX-505</t>
+          <t>WHPX 505</t>
         </is>
       </c>
       <c r="D1283" s="4" t="inlineStr"/>
@@ -47636,7 +47636,7 @@
       </c>
       <c r="C1284" s="2" t="inlineStr">
         <is>
-          <t>WHPX-505</t>
+          <t>WHPX 505</t>
         </is>
       </c>
       <c r="D1284" s="2" t="inlineStr"/>
@@ -47671,7 +47671,7 @@
       </c>
       <c r="C1285" s="4" t="inlineStr">
         <is>
-          <t>WHPX-505</t>
+          <t>WHPX 505</t>
         </is>
       </c>
       <c r="D1285" s="4" t="inlineStr"/>
@@ -47706,7 +47706,7 @@
       </c>
       <c r="C1286" s="2" t="inlineStr">
         <is>
-          <t>WHPX-505</t>
+          <t>WHPX 505</t>
         </is>
       </c>
       <c r="D1286" s="2" t="inlineStr"/>
@@ -47741,7 +47741,7 @@
       </c>
       <c r="C1287" s="4" t="inlineStr">
         <is>
-          <t>WHPX-407</t>
+          <t>WHPX 407</t>
         </is>
       </c>
       <c r="D1287" s="4" t="inlineStr"/>
@@ -47776,7 +47776,7 @@
       </c>
       <c r="C1288" s="2" t="inlineStr">
         <is>
-          <t>WHPX-407</t>
+          <t>WHPX 407</t>
         </is>
       </c>
       <c r="D1288" s="2" t="inlineStr"/>
@@ -47811,7 +47811,7 @@
       </c>
       <c r="C1289" s="4" t="inlineStr">
         <is>
-          <t>WHPX-407</t>
+          <t>WHPX 407</t>
         </is>
       </c>
       <c r="D1289" s="4" t="inlineStr"/>
@@ -47846,7 +47846,7 @@
       </c>
       <c r="C1290" s="2" t="inlineStr">
         <is>
-          <t>WHPX-407</t>
+          <t>WHPX 407</t>
         </is>
       </c>
       <c r="D1290" s="2" t="inlineStr"/>
@@ -47881,7 +47881,7 @@
       </c>
       <c r="C1291" s="4" t="inlineStr">
         <is>
-          <t>WHPX-407</t>
+          <t>WHPX 407</t>
         </is>
       </c>
       <c r="D1291" s="4" t="inlineStr"/>
@@ -47916,7 +47916,7 @@
       </c>
       <c r="C1292" s="2" t="inlineStr">
         <is>
-          <t>WHPX-409</t>
+          <t>WHPX 409</t>
         </is>
       </c>
       <c r="D1292" s="2" t="inlineStr"/>
@@ -47951,7 +47951,7 @@
       </c>
       <c r="C1293" s="4" t="inlineStr">
         <is>
-          <t>WHPX-409</t>
+          <t>WHPX 409</t>
         </is>
       </c>
       <c r="D1293" s="4" t="inlineStr"/>
@@ -47986,7 +47986,7 @@
       </c>
       <c r="C1294" s="2" t="inlineStr">
         <is>
-          <t>WHPX-409</t>
+          <t>WHPX 409</t>
         </is>
       </c>
       <c r="D1294" s="2" t="inlineStr"/>
@@ -48021,7 +48021,7 @@
       </c>
       <c r="C1295" s="4" t="inlineStr">
         <is>
-          <t>WHPX-409</t>
+          <t>WHPX 409</t>
         </is>
       </c>
       <c r="D1295" s="4" t="inlineStr"/>
@@ -48056,7 +48056,7 @@
       </c>
       <c r="C1296" s="2" t="inlineStr">
         <is>
-          <t>WHPX-409</t>
+          <t>WHPX 409</t>
         </is>
       </c>
       <c r="D1296" s="2" t="inlineStr"/>
@@ -48091,7 +48091,7 @@
       </c>
       <c r="C1297" s="4" t="inlineStr">
         <is>
-          <t>WHPX-410</t>
+          <t>WHPX 410</t>
         </is>
       </c>
       <c r="D1297" s="4" t="inlineStr"/>
@@ -48126,7 +48126,7 @@
       </c>
       <c r="C1298" s="2" t="inlineStr">
         <is>
-          <t>WHPX-410</t>
+          <t>WHPX 410</t>
         </is>
       </c>
       <c r="D1298" s="2" t="inlineStr"/>
@@ -48161,7 +48161,7 @@
       </c>
       <c r="C1299" s="4" t="inlineStr">
         <is>
-          <t>WHPX-410</t>
+          <t>WHPX 410</t>
         </is>
       </c>
       <c r="D1299" s="4" t="inlineStr"/>
@@ -48196,7 +48196,7 @@
       </c>
       <c r="C1300" s="2" t="inlineStr">
         <is>
-          <t>WHPX-410</t>
+          <t>WHPX 410</t>
         </is>
       </c>
       <c r="D1300" s="2" t="inlineStr"/>
@@ -48231,7 +48231,7 @@
       </c>
       <c r="C1301" s="4" t="inlineStr">
         <is>
-          <t>WHPX-410</t>
+          <t>WHPX 410</t>
         </is>
       </c>
       <c r="D1301" s="4" t="inlineStr"/>
@@ -48266,7 +48266,7 @@
       </c>
       <c r="C1302" s="2" t="inlineStr">
         <is>
-          <t>WHPX-413</t>
+          <t>WHPX 413</t>
         </is>
       </c>
       <c r="D1302" s="2" t="inlineStr"/>
@@ -48301,7 +48301,7 @@
       </c>
       <c r="C1303" s="4" t="inlineStr">
         <is>
-          <t>WHPX-413</t>
+          <t>WHPX 413</t>
         </is>
       </c>
       <c r="D1303" s="4" t="inlineStr"/>
@@ -48336,7 +48336,7 @@
       </c>
       <c r="C1304" s="2" t="inlineStr">
         <is>
-          <t>WHPX-413</t>
+          <t>WHPX 413</t>
         </is>
       </c>
       <c r="D1304" s="2" t="inlineStr"/>
@@ -48371,7 +48371,7 @@
       </c>
       <c r="C1305" s="4" t="inlineStr">
         <is>
-          <t>WHPX-413</t>
+          <t>WHPX 413</t>
         </is>
       </c>
       <c r="D1305" s="4" t="inlineStr"/>
@@ -48406,7 +48406,7 @@
       </c>
       <c r="C1306" s="2" t="inlineStr">
         <is>
-          <t>WHPX-413</t>
+          <t>WHPX 413</t>
         </is>
       </c>
       <c r="D1306" s="2" t="inlineStr"/>
@@ -48441,7 +48441,7 @@
       </c>
       <c r="C1307" s="4" t="inlineStr">
         <is>
-          <t>WHPX-507</t>
+          <t>WHPX 507</t>
         </is>
       </c>
       <c r="D1307" s="4" t="inlineStr"/>
@@ -48476,7 +48476,7 @@
       </c>
       <c r="C1308" s="2" t="inlineStr">
         <is>
-          <t>WHPX-507</t>
+          <t>WHPX 507</t>
         </is>
       </c>
       <c r="D1308" s="2" t="inlineStr"/>
@@ -48511,7 +48511,7 @@
       </c>
       <c r="C1309" s="4" t="inlineStr">
         <is>
-          <t>WHPX-507</t>
+          <t>WHPX 507</t>
         </is>
       </c>
       <c r="D1309" s="4" t="inlineStr"/>
@@ -48546,7 +48546,7 @@
       </c>
       <c r="C1310" s="2" t="inlineStr">
         <is>
-          <t>WHPX-507</t>
+          <t>WHPX 507</t>
         </is>
       </c>
       <c r="D1310" s="2" t="inlineStr"/>
@@ -48581,7 +48581,7 @@
       </c>
       <c r="C1311" s="4" t="inlineStr">
         <is>
-          <t>WHPX-507</t>
+          <t>WHPX 507</t>
         </is>
       </c>
       <c r="D1311" s="4" t="inlineStr"/>
@@ -48616,7 +48616,7 @@
       </c>
       <c r="C1312" s="2" t="inlineStr">
         <is>
-          <t>WHPX-508</t>
+          <t>WHPX 508</t>
         </is>
       </c>
       <c r="D1312" s="2" t="inlineStr"/>
@@ -48651,7 +48651,7 @@
       </c>
       <c r="C1313" s="4" t="inlineStr">
         <is>
-          <t>WHPX-508</t>
+          <t>WHPX 508</t>
         </is>
       </c>
       <c r="D1313" s="4" t="inlineStr"/>
@@ -48686,7 +48686,7 @@
       </c>
       <c r="C1314" s="2" t="inlineStr">
         <is>
-          <t>WHPX-508</t>
+          <t>WHPX 508</t>
         </is>
       </c>
       <c r="D1314" s="2" t="inlineStr"/>
@@ -48721,7 +48721,7 @@
       </c>
       <c r="C1315" s="4" t="inlineStr">
         <is>
-          <t>WHPX-508</t>
+          <t>WHPX 508</t>
         </is>
       </c>
       <c r="D1315" s="4" t="inlineStr"/>
@@ -48756,7 +48756,7 @@
       </c>
       <c r="C1316" s="2" t="inlineStr">
         <is>
-          <t>WHPX-508</t>
+          <t>WHPX 508</t>
         </is>
       </c>
       <c r="D1316" s="2" t="inlineStr"/>
@@ -48791,7 +48791,7 @@
       </c>
       <c r="C1317" s="4" t="inlineStr">
         <is>
-          <t>WHPX-513</t>
+          <t>WHPX 513</t>
         </is>
       </c>
       <c r="D1317" s="4" t="inlineStr"/>
@@ -48826,7 +48826,7 @@
       </c>
       <c r="C1318" s="2" t="inlineStr">
         <is>
-          <t>WHPX-513</t>
+          <t>WHPX 513</t>
         </is>
       </c>
       <c r="D1318" s="2" t="inlineStr"/>
@@ -48861,7 +48861,7 @@
       </c>
       <c r="C1319" s="4" t="inlineStr">
         <is>
-          <t>WHPX-513</t>
+          <t>WHPX 513</t>
         </is>
       </c>
       <c r="D1319" s="4" t="inlineStr"/>
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C1320" s="2" t="inlineStr">
         <is>
-          <t>WHPX-513</t>
+          <t>WHPX 513</t>
         </is>
       </c>
       <c r="D1320" s="2" t="inlineStr"/>
@@ -48931,7 +48931,7 @@
       </c>
       <c r="C1321" s="4" t="inlineStr">
         <is>
-          <t>WHPX-513</t>
+          <t>WHPX 513</t>
         </is>
       </c>
       <c r="D1321" s="4" t="inlineStr"/>
@@ -48966,7 +48966,7 @@
       </c>
       <c r="C1322" s="2" t="inlineStr">
         <is>
-          <t>SJ-E-all types</t>
+          <t>SJ-E all types</t>
         </is>
       </c>
       <c r="D1322" s="2" t="inlineStr"/>
@@ -49001,7 +49001,7 @@
       </c>
       <c r="C1323" s="4" t="inlineStr">
         <is>
-          <t>SJ-G-all types</t>
+          <t>SJ-G all types</t>
         </is>
       </c>
       <c r="D1323" s="4" t="inlineStr"/>
@@ -49071,7 +49071,7 @@
       </c>
       <c r="C1325" s="4" t="inlineStr">
         <is>
-          <t>OSA-7</t>
+          <t>OSA 7</t>
         </is>
       </c>
       <c r="D1325" s="4" t="inlineStr"/>
@@ -49106,7 +49106,7 @@
       </c>
       <c r="C1326" s="2" t="inlineStr">
         <is>
-          <t>OSA-7</t>
+          <t>OSA 7</t>
         </is>
       </c>
       <c r="D1326" s="2" t="inlineStr"/>
@@ -49141,7 +49141,7 @@
       </c>
       <c r="C1327" s="4" t="inlineStr">
         <is>
-          <t>OSA-20</t>
+          <t>OSA 20</t>
         </is>
       </c>
       <c r="D1327" s="4" t="inlineStr"/>
@@ -49176,7 +49176,7 @@
       </c>
       <c r="C1328" s="2" t="inlineStr">
         <is>
-          <t>OSA-35</t>
+          <t>OSA 35</t>
         </is>
       </c>
       <c r="D1328" s="2" t="inlineStr"/>
@@ -49211,7 +49211,7 @@
       </c>
       <c r="C1329" s="4" t="inlineStr">
         <is>
-          <t>OSB-20</t>
+          <t>OSB 20</t>
         </is>
       </c>
       <c r="D1329" s="4" t="inlineStr"/>
@@ -49246,7 +49246,7 @@
       </c>
       <c r="C1330" s="2" t="inlineStr">
         <is>
-          <t>OSB-30</t>
+          <t>OSB 30</t>
         </is>
       </c>
       <c r="D1330" s="2" t="inlineStr"/>
@@ -49281,7 +49281,7 @@
       </c>
       <c r="C1331" s="4" t="inlineStr">
         <is>
-          <t>OSB-35</t>
+          <t>OSB 35</t>
         </is>
       </c>
       <c r="D1331" s="4" t="inlineStr"/>
@@ -49316,7 +49316,7 @@
       </c>
       <c r="C1332" s="2" t="inlineStr">
         <is>
-          <t>OSC-4</t>
+          <t>OSC 4</t>
         </is>
       </c>
       <c r="D1332" s="2" t="inlineStr"/>
@@ -49351,7 +49351,7 @@
       </c>
       <c r="C1333" s="4" t="inlineStr">
         <is>
-          <t>OSC-4</t>
+          <t>OSC 4</t>
         </is>
       </c>
       <c r="D1333" s="4" t="inlineStr"/>
@@ -49386,7 +49386,7 @@
       </c>
       <c r="C1334" s="2" t="inlineStr">
         <is>
-          <t>OSC-5</t>
+          <t>OSC 5</t>
         </is>
       </c>
       <c r="D1334" s="2" t="inlineStr"/>
@@ -49421,7 +49421,7 @@
       </c>
       <c r="C1335" s="4" t="inlineStr">
         <is>
-          <t>OSC-5</t>
+          <t>OSC 5</t>
         </is>
       </c>
       <c r="D1335" s="4" t="inlineStr"/>
@@ -49456,7 +49456,7 @@
       </c>
       <c r="C1336" s="2" t="inlineStr">
         <is>
-          <t>OSC-15</t>
+          <t>OSC 15</t>
         </is>
       </c>
       <c r="D1336" s="2" t="inlineStr"/>
@@ -49491,7 +49491,7 @@
       </c>
       <c r="C1337" s="4" t="inlineStr">
         <is>
-          <t>OSC-18</t>
+          <t>OSC 18</t>
         </is>
       </c>
       <c r="D1337" s="4" t="inlineStr"/>
@@ -49526,7 +49526,7 @@
       </c>
       <c r="C1338" s="2" t="inlineStr">
         <is>
-          <t>OSC-25</t>
+          <t>OSC 25</t>
         </is>
       </c>
       <c r="D1338" s="2" t="inlineStr"/>
@@ -49561,7 +49561,7 @@
       </c>
       <c r="C1339" s="4" t="inlineStr">
         <is>
-          <t>OSC-30</t>
+          <t>OSC 30</t>
         </is>
       </c>
       <c r="D1339" s="4" t="inlineStr"/>
@@ -49596,7 +49596,7 @@
       </c>
       <c r="C1340" s="2" t="inlineStr">
         <is>
-          <t>OSC-40</t>
+          <t>OSC 40</t>
         </is>
       </c>
       <c r="D1340" s="2" t="inlineStr"/>
@@ -49631,7 +49631,7 @@
       </c>
       <c r="C1341" s="4" t="inlineStr">
         <is>
-          <t>OSC-50</t>
+          <t>OSC 50</t>
         </is>
       </c>
       <c r="D1341" s="4" t="inlineStr"/>
@@ -49666,7 +49666,7 @@
       </c>
       <c r="C1342" s="2" t="inlineStr">
         <is>
-          <t>OSD-all types</t>
+          <t>OSD all types</t>
         </is>
       </c>
       <c r="D1342" s="2" t="inlineStr"/>
@@ -49701,7 +49701,7 @@
       </c>
       <c r="C1343" s="4" t="inlineStr">
         <is>
-          <t>OSD-all types</t>
+          <t>OSD all types</t>
         </is>
       </c>
       <c r="D1343" s="4" t="inlineStr"/>
@@ -49736,7 +49736,7 @@
       </c>
       <c r="C1344" s="2" t="inlineStr">
         <is>
-          <t>OSE-all types</t>
+          <t>OSE all types</t>
         </is>
       </c>
       <c r="D1344" s="2" t="inlineStr"/>
@@ -49771,7 +49771,7 @@
       </c>
       <c r="C1345" s="4" t="inlineStr">
         <is>
-          <t>OSE-all types</t>
+          <t>OSE all types</t>
         </is>
       </c>
       <c r="D1345" s="4" t="inlineStr"/>
@@ -49806,7 +49806,7 @@
       </c>
       <c r="C1346" s="2" t="inlineStr">
         <is>
-          <t>OTA-2</t>
+          <t>OTA 2</t>
         </is>
       </c>
       <c r="D1346" s="2" t="inlineStr"/>
@@ -49841,7 +49841,7 @@
       </c>
       <c r="C1347" s="4" t="inlineStr">
         <is>
-          <t>OTA-7</t>
+          <t>OTA 7</t>
         </is>
       </c>
       <c r="D1347" s="4" t="inlineStr"/>
@@ -49876,7 +49876,7 @@
       </c>
       <c r="C1348" s="2" t="inlineStr">
         <is>
-          <t>OTA-14</t>
+          <t>OTA 14</t>
         </is>
       </c>
       <c r="D1348" s="2" t="inlineStr"/>
@@ -49911,7 +49911,7 @@
       </c>
       <c r="C1349" s="4" t="inlineStr">
         <is>
-          <t>OTA-14</t>
+          <t>OTA 14</t>
         </is>
       </c>
       <c r="D1349" s="4" t="inlineStr"/>
@@ -49946,7 +49946,7 @@
       </c>
       <c r="C1350" s="2" t="inlineStr">
         <is>
-          <t>OTA-14</t>
+          <t>OTA 14</t>
         </is>
       </c>
       <c r="D1350" s="2" t="inlineStr"/>
@@ -49981,7 +49981,7 @@
       </c>
       <c r="C1351" s="4" t="inlineStr">
         <is>
-          <t>OTA-18</t>
+          <t>OTA 18</t>
         </is>
       </c>
       <c r="D1351" s="4" t="inlineStr"/>
@@ -50016,7 +50016,7 @@
       </c>
       <c r="C1352" s="2" t="inlineStr">
         <is>
-          <t>OTA-30</t>
+          <t>OTA 30</t>
         </is>
       </c>
       <c r="D1352" s="2" t="inlineStr"/>
@@ -50051,7 +50051,7 @@
       </c>
       <c r="C1353" s="4" t="inlineStr">
         <is>
-          <t>OTB-1</t>
+          <t>OTB 1</t>
         </is>
       </c>
       <c r="D1353" s="4" t="inlineStr"/>
@@ -50086,7 +50086,7 @@
       </c>
       <c r="C1354" s="2" t="inlineStr">
         <is>
-          <t>OTB-1</t>
+          <t>OTB 1</t>
         </is>
       </c>
       <c r="D1354" s="2" t="inlineStr"/>
@@ -50121,7 +50121,7 @@
       </c>
       <c r="C1355" s="4" t="inlineStr">
         <is>
-          <t>OTB-3</t>
+          <t>OTB 3</t>
         </is>
       </c>
       <c r="D1355" s="4" t="inlineStr"/>
@@ -50156,7 +50156,7 @@
       </c>
       <c r="C1356" s="2" t="inlineStr">
         <is>
-          <t>OTB-3</t>
+          <t>OTB 3</t>
         </is>
       </c>
       <c r="D1356" s="2" t="inlineStr"/>
@@ -50191,7 +50191,7 @@
       </c>
       <c r="C1357" s="4" t="inlineStr">
         <is>
-          <t>OTB-9</t>
+          <t>OTB 9</t>
         </is>
       </c>
       <c r="D1357" s="4" t="inlineStr"/>
@@ -50226,7 +50226,7 @@
       </c>
       <c r="C1358" s="2" t="inlineStr">
         <is>
-          <t>OTB-9</t>
+          <t>OTB 9</t>
         </is>
       </c>
       <c r="D1358" s="2" t="inlineStr"/>
@@ -50261,7 +50261,7 @@
       </c>
       <c r="C1359" s="4" t="inlineStr">
         <is>
-          <t>OTB-18</t>
+          <t>OTB 18</t>
         </is>
       </c>
       <c r="D1359" s="4" t="inlineStr"/>
@@ -50296,7 +50296,7 @@
       </c>
       <c r="C1360" s="2" t="inlineStr">
         <is>
-          <t>OTB-35</t>
+          <t>OTB 35</t>
         </is>
       </c>
       <c r="D1360" s="2" t="inlineStr"/>
@@ -50331,7 +50331,7 @@
       </c>
       <c r="C1361" s="4" t="inlineStr">
         <is>
-          <t>OTC-all types</t>
+          <t>OTC all types</t>
         </is>
       </c>
       <c r="D1361" s="4" t="inlineStr"/>
@@ -50366,7 +50366,7 @@
       </c>
       <c r="C1362" s="2" t="inlineStr">
         <is>
-          <t>OTC-all types</t>
+          <t>OTC all types</t>
         </is>
       </c>
       <c r="D1362" s="2" t="inlineStr"/>

</xml_diff>